<commit_message>
docs(office): rebuild the TDP proposal, budget and deck from screenshots review
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -6,7 +6,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Milestones'!$A$1:$L$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$G$14</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -273,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -399,6 +402,87 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,7 +756,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
@@ -692,7 +776,7 @@
     <col width="8.710000000000001" customWidth="1" style="43" min="13" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40.5" customHeight="1" s="43">
+    <row r="1" ht="30" customHeight="1" s="43">
       <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Budget</t>
@@ -706,17 +790,17 @@
           <t>Milestone Timelines</t>
         </is>
       </c>
-      <c r="F1" s="44" t="n"/>
-      <c r="G1" s="44" t="n"/>
-      <c r="H1" s="45" t="n"/>
+      <c r="F1" s="57" t="n"/>
+      <c r="G1" s="57" t="n"/>
+      <c r="H1" s="58" t="n"/>
       <c r="I1" s="47" t="n"/>
-      <c r="J1" s="48" t="inlineStr">
+      <c r="J1" s="59" t="inlineStr">
         <is>
           <t>Tranche Disbursement Schedule</t>
         </is>
       </c>
-      <c r="K1" s="49" t="n"/>
-      <c r="L1" s="50" t="n"/>
+      <c r="K1" s="60" t="n"/>
+      <c r="L1" s="61" t="n"/>
       <c r="M1" s="12" t="n"/>
       <c r="N1" s="12" t="n"/>
       <c r="O1" s="12" t="n"/>
@@ -732,26 +816,26 @@
       <c r="Y1" s="12" t="n"/>
       <c r="Z1" s="12" t="n"/>
     </row>
-    <row r="2" ht="1.5" customHeight="1" s="43">
+    <row r="2" ht="30" customHeight="1" s="43">
       <c r="A2" s="51" t="n"/>
       <c r="B2" s="52" t="n"/>
       <c r="C2" s="53" t="n"/>
       <c r="E2" s="51" t="n"/>
-      <c r="F2" s="52" t="n"/>
-      <c r="G2" s="52" t="n"/>
-      <c r="H2" s="53" t="n"/>
+      <c r="F2" s="62" t="n"/>
+      <c r="G2" s="62" t="n"/>
+      <c r="H2" s="63" t="n"/>
       <c r="I2" s="54" t="n"/>
-      <c r="J2" s="21" t="inlineStr">
+      <c r="J2" s="64" t="inlineStr">
         <is>
           <t>Timeline</t>
         </is>
       </c>
-      <c r="K2" s="21" t="inlineStr">
+      <c r="K2" s="64" t="inlineStr">
         <is>
           <t>Amount to be released (INR) inclusive of GST</t>
         </is>
       </c>
-      <c r="L2" s="21" t="inlineStr">
+      <c r="L2" s="64" t="inlineStr">
         <is>
           <t>Milestone/Deliverables that will be completed  by the timeline</t>
         </is>
@@ -771,7 +855,7 @@
       <c r="Y2" s="12" t="n"/>
       <c r="Z2" s="12" t="n"/>
     </row>
-    <row r="3" ht="85.5" customHeight="1" s="43">
+    <row r="3" ht="30" customHeight="1" s="43">
       <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Sr. No.</t>
@@ -792,25 +876,25 @@
           <t>S No</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="F3" s="64" t="inlineStr">
         <is>
           <t>Milestone/Deliverable</t>
         </is>
       </c>
-      <c r="G3" s="23" t="inlineStr">
+      <c r="G3" s="65" t="inlineStr">
         <is>
           <t xml:space="preserve">Time Period </t>
         </is>
       </c>
-      <c r="H3" s="27" t="inlineStr">
+      <c r="H3" s="66" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
       <c r="I3" s="54" t="n"/>
-      <c r="J3" s="55" t="n"/>
-      <c r="K3" s="55" t="n"/>
-      <c r="L3" s="55" t="n"/>
+      <c r="J3" s="67" t="n"/>
+      <c r="K3" s="67" t="n"/>
+      <c r="L3" s="67" t="n"/>
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
@@ -826,7 +910,7 @@
       <c r="Y3" s="12" t="n"/>
       <c r="Z3" s="12" t="n"/>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="43">
+    <row r="4" ht="30" customHeight="1" s="43">
       <c r="A4" s="27" t="n">
         <v>1</v>
       </c>
@@ -841,31 +925,31 @@
       <c r="E4" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="66" t="inlineStr">
         <is>
-          <t>Project Beginning (T0)</t>
+          <t>Project beginning (T0)</t>
         </is>
       </c>
-      <c r="G4" s="27" t="inlineStr">
+      <c r="G4" s="66" t="inlineStr">
         <is>
           <t>T0</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
+      <c r="H4" s="68" t="inlineStr">
         <is>
           <t>Project plan, stakeholder alignment, BOM freeze</t>
         </is>
       </c>
       <c r="I4" s="54" t="n"/>
-      <c r="J4" s="27" t="inlineStr">
+      <c r="J4" s="66" t="inlineStr">
         <is>
           <t>Project Start Date (T0)</t>
         </is>
       </c>
-      <c r="K4" s="25" t="n">
+      <c r="K4" s="69" t="n">
         <v>8235</v>
       </c>
-      <c r="L4" s="27" t="inlineStr">
+      <c r="L4" s="66" t="inlineStr">
         <is>
           <t>M1 monitor build and dashboard</t>
         </is>
@@ -885,7 +969,7 @@
       <c r="Y4" s="12" t="n"/>
       <c r="Z4" s="12" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="30" customHeight="1" s="43">
       <c r="A5" s="27" t="n">
         <v>2</v>
       </c>
@@ -900,31 +984,31 @@
       <c r="E5" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="26" t="inlineStr">
+      <c r="F5" s="70" t="inlineStr">
         <is>
           <t>Milestone 1: Requirements and monitor prototype</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
+      <c r="G5" s="66" t="inlineStr">
         <is>
           <t>T0 + 2 months</t>
         </is>
       </c>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="H5" s="66" t="inlineStr">
         <is>
-          <t>M1 calibrated; TankScore validated; dashboard served from the tank unit</t>
+          <t>M1 calibrated; TankScore validated; dashboard from flash</t>
         </is>
       </c>
       <c r="I5" s="54" t="n"/>
-      <c r="J5" s="27" t="inlineStr">
+      <c r="J5" s="66" t="inlineStr">
         <is>
           <t>T0 + 06 months</t>
         </is>
       </c>
-      <c r="K5" s="25" t="n">
+      <c r="K5" s="69" t="n">
         <v>9415</v>
       </c>
-      <c r="L5" s="28" t="inlineStr">
+      <c r="L5" s="66" t="inlineStr">
         <is>
           <t>H1 home unit and C1 cleaning arm</t>
         </is>
@@ -944,7 +1028,7 @@
       <c r="Y5" s="12" t="n"/>
       <c r="Z5" s="12" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="30" customHeight="1" s="43">
       <c r="A6" s="27" t="n">
         <v>3</v>
       </c>
@@ -959,31 +1043,31 @@
       <c r="E6" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="26" t="inlineStr">
+      <c r="F6" s="70" t="inlineStr">
         <is>
           <t>Milestone 2: Home unit and dashboard</t>
         </is>
       </c>
-      <c r="G6" s="27" t="inlineStr">
+      <c r="G6" s="66" t="inlineStr">
         <is>
           <t>T0 + 4 months</t>
         </is>
       </c>
-      <c r="H6" s="27" t="inlineStr">
+      <c r="H6" s="66" t="inlineStr">
         <is>
-          <t>H1 TFT + pump control installed; dashboard and session log complete</t>
+          <t>H1 TFT + pump control; dashboard and session log</t>
         </is>
       </c>
       <c r="I6" s="54" t="n"/>
-      <c r="J6" s="27" t="inlineStr">
+      <c r="J6" s="66" t="inlineStr">
         <is>
           <t>T0 + 12 months</t>
         </is>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="K6" s="69" t="n">
         <v>5937</v>
       </c>
-      <c r="L6" s="28" t="inlineStr">
+      <c r="L6" s="66" t="inlineStr">
         <is>
           <t>Field validation and evidence pack</t>
         </is>
@@ -1003,7 +1087,7 @@
       <c r="Y6" s="12" t="n"/>
       <c r="Z6" s="12" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="30" customHeight="1" s="43">
       <c r="A7" s="27" t="n">
         <v>4</v>
       </c>
@@ -1018,31 +1102,31 @@
       <c r="E7" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="F7" s="26" t="inlineStr">
+      <c r="F7" s="70" t="inlineStr">
         <is>
           <t>Milestone 3: Cleaning arm</t>
         </is>
       </c>
-      <c r="G7" s="27" t="inlineStr">
+      <c r="G7" s="66" t="inlineStr">
         <is>
           <t>T0 + 8 months</t>
         </is>
       </c>
-      <c r="H7" s="27" t="inlineStr">
+      <c r="H7" s="66" t="inlineStr">
         <is>
-          <t>C1 built; three-ring cycle executed; coverage and repeatability measured</t>
+          <t>C1 built; three-ring cycle; coverage measured</t>
         </is>
       </c>
       <c r="I7" s="54" t="n"/>
-      <c r="J7" s="27" t="inlineStr">
+      <c r="J7" s="66" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="K7" s="25" t="n">
+      <c r="K7" s="69" t="n">
         <v>23587</v>
       </c>
-      <c r="L7" s="28" t="n"/>
+      <c r="L7" s="66" t="inlineStr"/>
       <c r="M7" s="12" t="n"/>
       <c r="N7" s="12" t="n"/>
       <c r="O7" s="12" t="n"/>
@@ -1058,7 +1142,7 @@
       <c r="Y7" s="12" t="n"/>
       <c r="Z7" s="12" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="30" customHeight="1" s="43">
       <c r="A8" s="27" t="n">
         <v>5</v>
       </c>
@@ -1073,25 +1157,25 @@
       <c r="E8" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="71" t="inlineStr">
         <is>
           <t>Milestone 4: Field validation</t>
         </is>
       </c>
-      <c r="G8" s="27" t="inlineStr">
+      <c r="G8" s="66" t="inlineStr">
         <is>
           <t>T0 + 12 months</t>
         </is>
       </c>
-      <c r="H8" s="27" t="inlineStr">
+      <c r="H8" s="66" t="inlineStr">
         <is>
-          <t>Three installations, 90 days of data, TRL 6+ evidence pack</t>
+          <t>Three installations, 90 days, TRL 6+ evidence</t>
         </is>
       </c>
       <c r="I8" s="54" t="n"/>
-      <c r="J8" s="27" t="n"/>
-      <c r="K8" s="32" t="n"/>
-      <c r="L8" s="28" t="n"/>
+      <c r="J8" s="66" t="n"/>
+      <c r="K8" s="72" t="n"/>
+      <c r="L8" s="66" t="n"/>
       <c r="M8" s="12" t="n"/>
       <c r="N8" s="12" t="n"/>
       <c r="O8" s="12" t="n"/>
@@ -1107,34 +1191,34 @@
       <c r="Y8" s="12" t="n"/>
       <c r="Z8" s="12" t="n"/>
     </row>
-    <row r="9" ht="34.5" customHeight="1" s="43">
+    <row r="9" ht="30" customHeight="1" s="43">
       <c r="A9" s="27" t="n">
         <v>6</v>
       </c>
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>Contingency (max @5% of 10)</t>
+          <t>Contingency (max 5%)</t>
         </is>
       </c>
       <c r="C9" s="25" t="n">
         <v>780</v>
       </c>
       <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27" t="inlineStr">
+      <c r="F9" s="66" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="G9" s="28" t="n"/>
-      <c r="H9" s="50" t="n"/>
+      <c r="G9" s="66" t="n"/>
+      <c r="H9" s="61" t="n"/>
       <c r="I9" s="54" t="n"/>
-      <c r="J9" s="27" t="inlineStr">
+      <c r="J9" s="66" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="K9" s="25" t="n"/>
-      <c r="L9" s="28" t="n"/>
+      <c r="K9" s="69" t="n"/>
+      <c r="L9" s="66" t="n"/>
       <c r="M9" s="12" t="n"/>
       <c r="N9" s="12" t="n"/>
       <c r="O9" s="12" t="n"/>
@@ -1150,7 +1234,7 @@
       <c r="Y9" s="12" t="n"/>
       <c r="Z9" s="12" t="n"/>
     </row>
-    <row r="10" ht="14.25" customHeight="1" s="43">
+    <row r="10" ht="30" customHeight="1" s="43">
       <c r="A10" s="27" t="n">
         <v>7</v>
       </c>
@@ -1163,13 +1247,13 @@
         <v>16380</v>
       </c>
       <c r="E10" s="36" t="n"/>
-      <c r="F10" s="37" t="n"/>
-      <c r="G10" s="38" t="n"/>
-      <c r="H10" s="39" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="74" t="n"/>
+      <c r="H10" s="75" t="n"/>
       <c r="I10" s="12" t="n"/>
-      <c r="J10" s="12" t="n"/>
-      <c r="K10" s="12" t="n"/>
-      <c r="L10" s="12" t="n"/>
+      <c r="J10" s="76" t="n"/>
+      <c r="K10" s="76" t="n"/>
+      <c r="L10" s="76" t="n"/>
       <c r="M10" s="12" t="n"/>
       <c r="N10" s="12" t="n"/>
       <c r="O10" s="12" t="n"/>
@@ -1185,7 +1269,7 @@
       <c r="Y10" s="12" t="n"/>
       <c r="Z10" s="12" t="n"/>
     </row>
-    <row r="11" ht="14.25" customHeight="1" s="43">
+    <row r="11" ht="30" customHeight="1" s="43">
       <c r="A11" s="27" t="n">
         <v>8</v>
       </c>
@@ -1198,13 +1282,13 @@
         <v>3276</v>
       </c>
       <c r="E11" s="40" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="41" t="n"/>
+      <c r="F11" s="76" t="n"/>
+      <c r="G11" s="76" t="n"/>
+      <c r="H11" s="77" t="n"/>
       <c r="I11" s="12" t="n"/>
-      <c r="J11" s="12" t="n"/>
-      <c r="K11" s="12" t="n"/>
-      <c r="L11" s="12" t="n"/>
+      <c r="J11" s="76" t="n"/>
+      <c r="K11" s="76" t="n"/>
+      <c r="L11" s="76" t="n"/>
       <c r="M11" s="12" t="n"/>
       <c r="N11" s="12" t="n"/>
       <c r="O11" s="12" t="n"/>
@@ -1220,26 +1304,26 @@
       <c r="Y11" s="12" t="n"/>
       <c r="Z11" s="12" t="n"/>
     </row>
-    <row r="12" ht="78" customHeight="1" s="43">
+    <row r="12" ht="30" customHeight="1" s="43">
       <c r="A12" s="27" t="n">
         <v>9</v>
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>Faculty Fee (inclusive of all overheads/ institute share etc) @maximum of 20%of total project value</t>
+          <t>Faculty fee (max 20%)</t>
         </is>
       </c>
       <c r="C12" s="25" t="n">
         <v>3931</v>
       </c>
       <c r="E12" s="40" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="41" t="n"/>
+      <c r="F12" s="76" t="n"/>
+      <c r="G12" s="76" t="n"/>
+      <c r="H12" s="77" t="n"/>
       <c r="I12" s="12" t="n"/>
-      <c r="J12" s="12" t="n"/>
-      <c r="K12" s="12" t="n"/>
-      <c r="L12" s="12" t="n"/>
+      <c r="J12" s="76" t="n"/>
+      <c r="K12" s="76" t="n"/>
+      <c r="L12" s="76" t="n"/>
       <c r="M12" s="12" t="n"/>
       <c r="N12" s="12" t="n"/>
       <c r="O12" s="12" t="n"/>
@@ -1255,7 +1339,7 @@
       <c r="Y12" s="12" t="n"/>
       <c r="Z12" s="12" t="n"/>
     </row>
-    <row r="13" ht="14.25" customHeight="1" s="43">
+    <row r="13" ht="30" customHeight="1" s="43">
       <c r="A13" s="27" t="n">
         <v>10</v>
       </c>
@@ -1268,13 +1352,13 @@
         <v>23587</v>
       </c>
       <c r="E13" s="40" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="40" t="n"/>
+      <c r="F13" s="76" t="n"/>
+      <c r="G13" s="76" t="n"/>
+      <c r="H13" s="78" t="n"/>
       <c r="I13" s="12" t="n"/>
-      <c r="J13" s="12" t="n"/>
-      <c r="K13" s="12" t="n"/>
-      <c r="L13" s="12" t="n"/>
+      <c r="J13" s="76" t="n"/>
+      <c r="K13" s="76" t="n"/>
+      <c r="L13" s="76" t="n"/>
       <c r="M13" s="12" t="n"/>
       <c r="N13" s="12" t="n"/>
       <c r="O13" s="12" t="n"/>
@@ -1290,7 +1374,7 @@
       <c r="Y13" s="12" t="n"/>
       <c r="Z13" s="12" t="n"/>
     </row>
-    <row r="14" ht="14.25" customHeight="1" s="43">
+    <row r="14" ht="30" customHeight="1" s="43">
       <c r="A14" s="27" t="n">
         <v>11</v>
       </c>
@@ -1303,13 +1387,13 @@
         <v>0</v>
       </c>
       <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
-      <c r="H14" s="12" t="n"/>
+      <c r="F14" s="76" t="n"/>
+      <c r="G14" s="76" t="n"/>
+      <c r="H14" s="76" t="n"/>
       <c r="I14" s="12" t="n"/>
-      <c r="J14" s="12" t="n"/>
-      <c r="K14" s="12" t="n"/>
-      <c r="L14" s="12" t="n"/>
+      <c r="J14" s="76" t="n"/>
+      <c r="K14" s="76" t="n"/>
+      <c r="L14" s="76" t="n"/>
       <c r="M14" s="12" t="n"/>
       <c r="N14" s="12" t="n"/>
       <c r="O14" s="12" t="n"/>
@@ -1325,7 +1409,7 @@
       <c r="Y14" s="12" t="n"/>
       <c r="Z14" s="12" t="n"/>
     </row>
-    <row r="15" ht="14.25" customHeight="1" s="43">
+    <row r="15" ht="30" customHeight="1" s="43">
       <c r="A15" s="27" t="n">
         <v>12</v>
       </c>
@@ -1339,13 +1423,13 @@
       </c>
       <c r="D15" s="56" t="n"/>
       <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="12" t="n"/>
-      <c r="H15" s="12" t="n"/>
+      <c r="F15" s="76" t="n"/>
+      <c r="G15" s="76" t="n"/>
+      <c r="H15" s="76" t="n"/>
       <c r="I15" s="12" t="n"/>
-      <c r="J15" s="12" t="n"/>
-      <c r="K15" s="12" t="n"/>
-      <c r="L15" s="12" t="n"/>
+      <c r="J15" s="76" t="n"/>
+      <c r="K15" s="76" t="n"/>
+      <c r="L15" s="76" t="n"/>
       <c r="M15" s="12" t="n"/>
       <c r="N15" s="12" t="n"/>
       <c r="O15" s="12" t="n"/>
@@ -28953,8 +29037,9 @@
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="L2:L3"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -28962,9 +29047,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1002"/>
+  <dimension ref="A1:Z997"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="43" min="1" max="2"/>
@@ -28976,14 +29061,14 @@
     <col width="8.710000000000001" customWidth="1" style="43" min="8" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" s="43">
+    <row r="1" ht="26" customHeight="1" s="43">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
+      <c r="B1" s="79" t="n"/>
+      <c r="C1" s="79" t="n"/>
+      <c r="D1" s="79" t="n"/>
+      <c r="E1" s="79" t="n"/>
+      <c r="F1" s="79" t="n"/>
+      <c r="G1" s="79" t="n"/>
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
@@ -29004,17 +29089,17 @@
       <c r="Y1" s="1" t="n"/>
       <c r="Z1" s="1" t="n"/>
     </row>
-    <row r="2" ht="14.25" customHeight="1" s="43">
+    <row r="2" ht="26" customHeight="1" s="43">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
+      <c r="B2" s="79" t="n"/>
+      <c r="C2" s="79" t="n"/>
+      <c r="D2" s="79" t="n"/>
+      <c r="E2" s="79" t="n"/>
+      <c r="F2" s="79" t="n"/>
+      <c r="G2" s="79" t="n"/>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Grant Total (INR) - Full proposal build: 23,587</t>
+          <t>Grant total: INR 23,587</t>
         </is>
       </c>
       <c r="I2" s="1" t="n"/>
@@ -29036,28 +29121,31 @@
       <c r="Y2" s="1" t="n"/>
       <c r="Z2" s="1" t="n"/>
     </row>
-    <row r="3">
+    <row r="3" ht="26" customHeight="1" s="43">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="80" t="inlineStr">
         <is>
           <t>Milestone Expenditure Sheet</t>
         </is>
       </c>
-      <c r="C3" s="49" t="n"/>
-      <c r="D3" s="50" t="n"/>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="C3" s="60" t="n"/>
+      <c r="D3" s="61" t="n"/>
+      <c r="E3" s="80" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Tranche 1 Amount in Rs. XXXXXX</t>
+          <t>Tranche 1
+8,235</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="80" t="inlineStr">
         <is>
-          <t>Tranche 2 Amount in Rs. XXXXXX</t>
+          <t>Tranche 2
+9,415</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="80" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Tranche 3 Amount in Rs. XXXXXX</t>
+          <t>Tranche 3
+5,937</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -29084,37 +29172,37 @@
       <c r="Y3" s="1" t="n"/>
       <c r="Z3" s="1" t="n"/>
     </row>
-    <row r="4" ht="14.25" customHeight="1" s="43">
+    <row r="4" ht="26" customHeight="1" s="43">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="80" t="inlineStr">
         <is>
           <t>Sr.No.</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="80" t="inlineStr">
         <is>
           <t>Expenditure Heads</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="80" t="inlineStr">
         <is>
           <t>Total Funding
 Amount</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="80" t="inlineStr">
         <is>
           <t>Budgeted
 Amount</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="80" t="inlineStr">
         <is>
           <t>Budgeted
 Amount</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="80" t="inlineStr">
         <is>
           <t>Budgeted
 Amount</t>
@@ -29140,20 +29228,22 @@
       <c r="Y4" s="1" t="n"/>
       <c r="Z4" s="1" t="n"/>
     </row>
-    <row r="5" ht="14.25" customHeight="1" s="43">
+    <row r="5" ht="26" customHeight="1" s="43">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manpower </t>
+          <t>Manpower</t>
         </is>
       </c>
-      <c r="D5" s="22" t="n"/>
-      <c r="E5" s="22" t="n"/>
-      <c r="F5" s="22" t="n"/>
-      <c r="G5" s="22" t="n"/>
+      <c r="D5" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="81" t="n"/>
+      <c r="F5" s="81" t="n"/>
+      <c r="G5" s="81" t="n"/>
       <c r="H5" s="1" t="n"/>
       <c r="I5" s="1" t="n"/>
       <c r="J5" s="1" t="n"/>
@@ -29174,20 +29264,22 @@
       <c r="Y5" s="1" t="n"/>
       <c r="Z5" s="1" t="n"/>
     </row>
-    <row r="6" ht="14.25" customHeight="1" s="43">
+    <row r="6" ht="26" customHeight="1" s="43">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipment </t>
+          <t>Equipment (Exclusive of GST)</t>
         </is>
       </c>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="22" t="n"/>
-      <c r="F6" s="22" t="n"/>
-      <c r="G6" s="22" t="n"/>
+      <c r="D6" s="82" t="n">
+        <v>15600</v>
+      </c>
+      <c r="E6" s="81" t="n"/>
+      <c r="F6" s="81" t="n"/>
+      <c r="G6" s="81" t="n"/>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="n"/>
@@ -29208,20 +29300,22 @@
       <c r="Y6" s="1" t="n"/>
       <c r="Z6" s="1" t="n"/>
     </row>
-    <row r="7" ht="14.25" customHeight="1" s="43">
+    <row r="7" ht="26" customHeight="1" s="43">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consumables </t>
+          <t>Contingency (max 5%)</t>
         </is>
       </c>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
+      <c r="D7" s="82" t="n">
+        <v>780</v>
+      </c>
+      <c r="E7" s="81" t="n"/>
+      <c r="F7" s="81" t="n"/>
+      <c r="G7" s="81" t="n"/>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
       <c r="J7" s="1" t="n"/>
@@ -29242,20 +29336,22 @@
       <c r="Y7" s="1" t="n"/>
       <c r="Z7" s="1" t="n"/>
     </row>
-    <row r="8" ht="14.25" customHeight="1" s="43">
+    <row r="8" ht="26" customHeight="1" s="43">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel </t>
+          <t>Sub total</t>
         </is>
       </c>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
+      <c r="D8" s="82" t="n">
+        <v>16380</v>
+      </c>
+      <c r="E8" s="81" t="n"/>
+      <c r="F8" s="81" t="n"/>
+      <c r="G8" s="81" t="n"/>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
       <c r="J8" s="1" t="n"/>
@@ -29276,20 +29372,22 @@
       <c r="Y8" s="1" t="n"/>
       <c r="Z8" s="1" t="n"/>
     </row>
-    <row r="9" ht="14.25" customHeight="1" s="43">
+    <row r="9" ht="26" customHeight="1" s="43">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="64" t="inlineStr">
         <is>
-          <t>Miscellaneous expenses</t>
+          <t>Overhead (max 20%)</t>
         </is>
       </c>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="22" t="n"/>
-      <c r="G9" s="22" t="n"/>
+      <c r="D9" s="82" t="n">
+        <v>3276</v>
+      </c>
+      <c r="E9" s="81" t="n"/>
+      <c r="F9" s="81" t="n"/>
+      <c r="G9" s="81" t="n"/>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
       <c r="J9" s="1" t="n"/>
@@ -29310,22 +29408,22 @@
       <c r="Y9" s="1" t="n"/>
       <c r="Z9" s="1" t="n"/>
     </row>
-    <row r="10" ht="14.25" customHeight="1" s="43">
+    <row r="10" ht="26" customHeight="1" s="43">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="66" t="inlineStr">
         <is>
-          <t>Manpower</t>
+          <t>Faculty Fee (max 20%)</t>
         </is>
       </c>
-      <c r="D10" s="22" t="n">
-        <v>0</v>
+      <c r="D10" s="82" t="n">
+        <v>3931</v>
       </c>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="22" t="n"/>
-      <c r="G10" s="22" t="n"/>
+      <c r="E10" s="81" t="n"/>
+      <c r="F10" s="81" t="n"/>
+      <c r="G10" s="81" t="n"/>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
       <c r="J10" s="1" t="n"/>
@@ -29346,22 +29444,22 @@
       <c r="Y10" s="1" t="n"/>
       <c r="Z10" s="1" t="n"/>
     </row>
-    <row r="11" ht="14.25" customHeight="1" s="43">
+    <row r="11" ht="26" customHeight="1" s="43">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="81" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="64" t="inlineStr">
         <is>
-          <t>Equipment (Exclusive of GST)</t>
+          <t>Total (7+8+9)</t>
         </is>
       </c>
-      <c r="D11" s="22" t="n">
-        <v>15600</v>
+      <c r="D11" s="82" t="n">
+        <v>23587</v>
       </c>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="22" t="n"/>
-      <c r="G11" s="22" t="n"/>
+      <c r="E11" s="81" t="n"/>
+      <c r="F11" s="81" t="n"/>
+      <c r="G11" s="81" t="n"/>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="1" t="n"/>
@@ -29382,22 +29480,14 @@
       <c r="Y11" s="1" t="n"/>
       <c r="Z11" s="1" t="n"/>
     </row>
-    <row r="12" ht="14.25" customHeight="1" s="43">
+    <row r="12" ht="26" customHeight="1" s="43">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="22" t="n">
-        <v>8</v>
-      </c>
-      <c r="C12" s="27" t="inlineStr">
-        <is>
-          <t>Contingency (max 5%)</t>
-        </is>
-      </c>
-      <c r="D12" s="22" t="n">
-        <v>780</v>
-      </c>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="22" t="n"/>
+      <c r="B12" s="81" t="n"/>
+      <c r="C12" s="81" t="n"/>
+      <c r="D12" s="81" t="n"/>
+      <c r="E12" s="81" t="n"/>
+      <c r="F12" s="81" t="n"/>
+      <c r="G12" s="81" t="n"/>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
       <c r="J12" s="1" t="n"/>
@@ -29418,22 +29508,18 @@
       <c r="Y12" s="1" t="n"/>
       <c r="Z12" s="1" t="n"/>
     </row>
-    <row r="13" ht="14.25" customHeight="1" s="43">
+    <row r="13" ht="20" customHeight="1" s="43">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="C13" s="27" t="inlineStr">
+      <c r="B13" s="83" t="inlineStr">
         <is>
-          <t>Sub total</t>
+          <t>80% of the tranche fund should be utilized before claiming for the next tranche.</t>
         </is>
       </c>
-      <c r="D13" s="22" t="n">
-        <v>16380</v>
-      </c>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="22" t="n"/>
-      <c r="G13" s="22" t="n"/>
+      <c r="C13" s="60" t="n"/>
+      <c r="D13" s="60" t="n"/>
+      <c r="E13" s="60" t="n"/>
+      <c r="F13" s="61" t="n"/>
+      <c r="G13" s="81" t="n"/>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
       <c r="J13" s="1" t="n"/>
@@ -29454,22 +29540,14 @@
       <c r="Y13" s="1" t="n"/>
       <c r="Z13" s="1" t="n"/>
     </row>
-    <row r="14" ht="14.25" customHeight="1" s="43">
+    <row r="14" ht="26" customHeight="1" s="43">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="22" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" s="21" t="inlineStr">
-        <is>
-          <t>Overhead (max 20%)</t>
-        </is>
-      </c>
-      <c r="D14" s="22" t="n">
-        <v>3276</v>
-      </c>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="22" t="n"/>
-      <c r="G14" s="22" t="n"/>
+      <c r="B14" s="79" t="n"/>
+      <c r="C14" s="79" t="n"/>
+      <c r="D14" s="79" t="n"/>
+      <c r="E14" s="79" t="n"/>
+      <c r="F14" s="79" t="n"/>
+      <c r="G14" s="79" t="n"/>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
       <c r="J14" s="1" t="n"/>
@@ -29490,22 +29568,14 @@
       <c r="Y14" s="1" t="n"/>
       <c r="Z14" s="1" t="n"/>
     </row>
-    <row r="15" ht="14.25" customHeight="1" s="43">
+    <row r="15" ht="26" customHeight="1" s="43">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="22" t="n">
-        <v>11</v>
-      </c>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t>Faculty Fee (max 20%)</t>
-        </is>
-      </c>
-      <c r="D15" s="22" t="n">
-        <v>3931</v>
-      </c>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
+      <c r="B15" s="79" t="n"/>
+      <c r="C15" s="79" t="n"/>
+      <c r="D15" s="79" t="n"/>
+      <c r="E15" s="79" t="n"/>
+      <c r="F15" s="79" t="n"/>
+      <c r="G15" s="79" t="n"/>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
       <c r="J15" s="1" t="n"/>
@@ -29526,22 +29596,14 @@
       <c r="Y15" s="1" t="n"/>
       <c r="Z15" s="1" t="n"/>
     </row>
-    <row r="16" ht="14.25" customHeight="1" s="43">
+    <row r="16" ht="26" customHeight="1" s="43">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="29" t="n">
-        <v>12</v>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>Total (7+8+9)</t>
-        </is>
-      </c>
-      <c r="D16" s="30" t="n">
-        <v>23587</v>
-      </c>
-      <c r="E16" s="30" t="n"/>
-      <c r="F16" s="30" t="n"/>
-      <c r="G16" s="22" t="n"/>
+      <c r="B16" s="79" t="n"/>
+      <c r="C16" s="79" t="n"/>
+      <c r="D16" s="79" t="n"/>
+      <c r="E16" s="79" t="n"/>
+      <c r="F16" s="79" t="n"/>
+      <c r="G16" s="79" t="n"/>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
@@ -29562,14 +29624,14 @@
       <c r="Y16" s="1" t="n"/>
       <c r="Z16" s="1" t="n"/>
     </row>
-    <row r="17" ht="14.25" customHeight="1" s="43">
+    <row r="17" ht="26" customHeight="1" s="43">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="30" t="n"/>
-      <c r="C17" s="30" t="n"/>
-      <c r="D17" s="30" t="n"/>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="30" t="n"/>
-      <c r="G17" s="22" t="n"/>
+      <c r="B17" s="79" t="n"/>
+      <c r="C17" s="79" t="n"/>
+      <c r="D17" s="79" t="n"/>
+      <c r="E17" s="79" t="n"/>
+      <c r="F17" s="79" t="n"/>
+      <c r="G17" s="79" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
       <c r="J17" s="1" t="n"/>
@@ -29592,16 +29654,12 @@
     </row>
     <row r="18" ht="14.25" customHeight="1" s="43">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>80% of the tranche fund should be utilized before claiming for the next tranche.</t>
-        </is>
-      </c>
-      <c r="C18" s="49" t="n"/>
-      <c r="D18" s="49" t="n"/>
-      <c r="E18" s="49" t="n"/>
-      <c r="F18" s="50" t="n"/>
-      <c r="G18" s="22" t="n"/>
+      <c r="B18" s="1" t="n"/>
+      <c r="C18" s="1" t="n"/>
+      <c r="D18" s="1" t="n"/>
+      <c r="E18" s="1" t="n"/>
+      <c r="F18" s="1" t="n"/>
+      <c r="G18" s="1" t="n"/>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
       <c r="J18" s="1" t="n"/>
@@ -57034,152 +57092,18 @@
       <c r="Y997" s="1" t="n"/>
       <c r="Z997" s="1" t="n"/>
     </row>
-    <row r="998" ht="14.25" customHeight="1" s="43">
-      <c r="A998" s="1" t="n"/>
-      <c r="B998" s="1" t="n"/>
-      <c r="C998" s="1" t="n"/>
-      <c r="D998" s="1" t="n"/>
-      <c r="E998" s="1" t="n"/>
-      <c r="F998" s="1" t="n"/>
-      <c r="G998" s="1" t="n"/>
-      <c r="H998" s="1" t="n"/>
-      <c r="I998" s="1" t="n"/>
-      <c r="J998" s="1" t="n"/>
-      <c r="K998" s="1" t="n"/>
-      <c r="L998" s="1" t="n"/>
-      <c r="M998" s="1" t="n"/>
-      <c r="N998" s="1" t="n"/>
-      <c r="O998" s="1" t="n"/>
-      <c r="P998" s="1" t="n"/>
-      <c r="Q998" s="1" t="n"/>
-      <c r="R998" s="1" t="n"/>
-      <c r="S998" s="1" t="n"/>
-      <c r="T998" s="1" t="n"/>
-      <c r="U998" s="1" t="n"/>
-      <c r="V998" s="1" t="n"/>
-      <c r="W998" s="1" t="n"/>
-      <c r="X998" s="1" t="n"/>
-      <c r="Y998" s="1" t="n"/>
-      <c r="Z998" s="1" t="n"/>
-    </row>
-    <row r="999" ht="14.25" customHeight="1" s="43">
-      <c r="A999" s="1" t="n"/>
-      <c r="B999" s="1" t="n"/>
-      <c r="C999" s="1" t="n"/>
-      <c r="D999" s="1" t="n"/>
-      <c r="E999" s="1" t="n"/>
-      <c r="F999" s="1" t="n"/>
-      <c r="G999" s="1" t="n"/>
-      <c r="H999" s="1" t="n"/>
-      <c r="I999" s="1" t="n"/>
-      <c r="J999" s="1" t="n"/>
-      <c r="K999" s="1" t="n"/>
-      <c r="L999" s="1" t="n"/>
-      <c r="M999" s="1" t="n"/>
-      <c r="N999" s="1" t="n"/>
-      <c r="O999" s="1" t="n"/>
-      <c r="P999" s="1" t="n"/>
-      <c r="Q999" s="1" t="n"/>
-      <c r="R999" s="1" t="n"/>
-      <c r="S999" s="1" t="n"/>
-      <c r="T999" s="1" t="n"/>
-      <c r="U999" s="1" t="n"/>
-      <c r="V999" s="1" t="n"/>
-      <c r="W999" s="1" t="n"/>
-      <c r="X999" s="1" t="n"/>
-      <c r="Y999" s="1" t="n"/>
-      <c r="Z999" s="1" t="n"/>
-    </row>
-    <row r="1000" ht="14.25" customHeight="1" s="43">
-      <c r="A1000" s="1" t="n"/>
-      <c r="B1000" s="1" t="n"/>
-      <c r="C1000" s="1" t="n"/>
-      <c r="D1000" s="1" t="n"/>
-      <c r="E1000" s="1" t="n"/>
-      <c r="F1000" s="1" t="n"/>
-      <c r="G1000" s="1" t="n"/>
-      <c r="H1000" s="1" t="n"/>
-      <c r="I1000" s="1" t="n"/>
-      <c r="J1000" s="1" t="n"/>
-      <c r="K1000" s="1" t="n"/>
-      <c r="L1000" s="1" t="n"/>
-      <c r="M1000" s="1" t="n"/>
-      <c r="N1000" s="1" t="n"/>
-      <c r="O1000" s="1" t="n"/>
-      <c r="P1000" s="1" t="n"/>
-      <c r="Q1000" s="1" t="n"/>
-      <c r="R1000" s="1" t="n"/>
-      <c r="S1000" s="1" t="n"/>
-      <c r="T1000" s="1" t="n"/>
-      <c r="U1000" s="1" t="n"/>
-      <c r="V1000" s="1" t="n"/>
-      <c r="W1000" s="1" t="n"/>
-      <c r="X1000" s="1" t="n"/>
-      <c r="Y1000" s="1" t="n"/>
-      <c r="Z1000" s="1" t="n"/>
-    </row>
-    <row r="1001" ht="14.25" customHeight="1" s="43">
-      <c r="A1001" s="1" t="n"/>
-      <c r="B1001" s="1" t="n"/>
-      <c r="C1001" s="1" t="n"/>
-      <c r="D1001" s="1" t="n"/>
-      <c r="E1001" s="1" t="n"/>
-      <c r="F1001" s="1" t="n"/>
-      <c r="G1001" s="1" t="n"/>
-      <c r="H1001" s="1" t="n"/>
-      <c r="I1001" s="1" t="n"/>
-      <c r="J1001" s="1" t="n"/>
-      <c r="K1001" s="1" t="n"/>
-      <c r="L1001" s="1" t="n"/>
-      <c r="M1001" s="1" t="n"/>
-      <c r="N1001" s="1" t="n"/>
-      <c r="O1001" s="1" t="n"/>
-      <c r="P1001" s="1" t="n"/>
-      <c r="Q1001" s="1" t="n"/>
-      <c r="R1001" s="1" t="n"/>
-      <c r="S1001" s="1" t="n"/>
-      <c r="T1001" s="1" t="n"/>
-      <c r="U1001" s="1" t="n"/>
-      <c r="V1001" s="1" t="n"/>
-      <c r="W1001" s="1" t="n"/>
-      <c r="X1001" s="1" t="n"/>
-      <c r="Y1001" s="1" t="n"/>
-      <c r="Z1001" s="1" t="n"/>
-    </row>
-    <row r="1002" ht="14.25" customHeight="1" s="43">
-      <c r="A1002" s="1" t="n"/>
-      <c r="B1002" s="1" t="n"/>
-      <c r="C1002" s="1" t="n"/>
-      <c r="D1002" s="1" t="n"/>
-      <c r="E1002" s="1" t="n"/>
-      <c r="F1002" s="1" t="n"/>
-      <c r="G1002" s="1" t="n"/>
-      <c r="H1002" s="1" t="n"/>
-      <c r="I1002" s="1" t="n"/>
-      <c r="J1002" s="1" t="n"/>
-      <c r="K1002" s="1" t="n"/>
-      <c r="L1002" s="1" t="n"/>
-      <c r="M1002" s="1" t="n"/>
-      <c r="N1002" s="1" t="n"/>
-      <c r="O1002" s="1" t="n"/>
-      <c r="P1002" s="1" t="n"/>
-      <c r="Q1002" s="1" t="n"/>
-      <c r="R1002" s="1" t="n"/>
-      <c r="S1002" s="1" t="n"/>
-      <c r="T1002" s="1" t="n"/>
-      <c r="U1002" s="1" t="n"/>
-      <c r="V1002" s="1" t="n"/>
-      <c r="W1002" s="1" t="n"/>
-      <c r="X1002" s="1" t="n"/>
-      <c r="Y1002" s="1" t="n"/>
-      <c r="Z1002" s="1" t="n"/>
-    </row>
+    <row r="998" ht="14.25" customHeight="1" s="43"/>
+    <row r="999" ht="14.25" customHeight="1" s="43"/>
+    <row r="1000" ht="14.25" customHeight="1" s="43"/>
+    <row r="1001" ht="14.25" customHeight="1" s="43"/>
+    <row r="1002" ht="14.25" customHeight="1" s="43"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B18:F18"/>
   </mergeCells>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(office): rewrite the TDP copy and rebuild the deck layout
The deck was a list of one-line claims with no setup, so a reader landing mid-deck had no context. Every slide now opens with a takeaway, carries three or four labelled cards, and closes with a callout. The narrative adds what is already built and folds market into impact.

The proposal gets dot-leader contents with page numbers, consistent table widths, right-aligned amounts, and no orphaned headings. The budget workbook is rebuilt as clean tables with a readable summary sheet.

The specification is corrected to the shipped firmware: ESP8266 on M1, weights 40/25/25/10 with level unscored, three score bands, and a BOM that matches the grant budget.
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -8,7 +8,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Milestones'!$A$1:$L$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$G$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$D$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -68,8 +68,47 @@
       <color rgb="FF6D9EEB"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002E74B5"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -82,8 +121,23 @@
         <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E74B5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF3F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border/>
     <border>
       <left style="thin">
@@ -272,11 +326,25 @@
         <color rgb="FF000000"/>
       </right>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C3D3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C3D3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -402,86 +470,77 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -761,46 +820,39 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="8.710000000000001" customWidth="1" style="43" min="1" max="1"/>
-    <col width="27.43" customWidth="1" style="43" min="2" max="2"/>
-    <col width="21.71" customWidth="1" style="43" min="3" max="3"/>
-    <col width="1.86" customWidth="1" style="43" min="4" max="4"/>
-    <col width="8.710000000000001" customWidth="1" style="43" min="5" max="5"/>
-    <col width="44.86" customWidth="1" style="43" min="6" max="6"/>
-    <col width="20.86" customWidth="1" style="43" min="7" max="7"/>
-    <col width="27" customWidth="1" style="43" min="8" max="8"/>
-    <col width="1.43" customWidth="1" style="43" min="9" max="9"/>
-    <col width="36" customWidth="1" style="43" min="10" max="10"/>
-    <col width="21.14" customWidth="1" style="43" min="11" max="11"/>
-    <col width="34" customWidth="1" style="43" min="12" max="12"/>
+    <col width="7" customWidth="1" style="43" min="1" max="1"/>
+    <col width="29" customWidth="1" style="43" min="2" max="2"/>
+    <col width="13" customWidth="1" style="43" min="3" max="3"/>
+    <col width="2.5" customWidth="1" style="43" min="4" max="4"/>
+    <col width="5.5" customWidth="1" style="43" min="5" max="5"/>
+    <col width="31" customWidth="1" style="43" min="6" max="6"/>
+    <col width="15" customWidth="1" style="43" min="7" max="7"/>
+    <col width="34" customWidth="1" style="43" min="8" max="8"/>
+    <col width="2.5" customWidth="1" style="43" min="9" max="9"/>
+    <col width="19" customWidth="1" style="43" min="10" max="10"/>
+    <col width="14" customWidth="1" style="43" min="11" max="11"/>
+    <col width="38" customWidth="1" style="43" min="12" max="12"/>
     <col width="8.710000000000001" customWidth="1" style="43" min="13" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="43">
-      <c r="A1" s="21" t="inlineStr">
+    <row r="1" ht="26" customHeight="1" s="43">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="B1" s="44" t="n"/>
-      <c r="C1" s="45" t="n"/>
-      <c r="D1" s="46" t="n"/>
-      <c r="E1" s="21" t="inlineStr">
+      <c r="D1" s="40" t="n"/>
+      <c r="E1" s="57" t="inlineStr">
         <is>
           <t>Milestone Timelines</t>
         </is>
       </c>
-      <c r="F1" s="57" t="n"/>
-      <c r="G1" s="57" t="n"/>
-      <c r="H1" s="58" t="n"/>
-      <c r="I1" s="47" t="n"/>
-      <c r="J1" s="59" t="inlineStr">
+      <c r="I1" s="12" t="n"/>
+      <c r="J1" s="57" t="inlineStr">
         <is>
           <t>Tranche Disbursement Schedule</t>
         </is>
       </c>
-      <c r="K1" s="60" t="n"/>
-      <c r="L1" s="61" t="n"/>
       <c r="M1" s="12" t="n"/>
       <c r="N1" s="12" t="n"/>
       <c r="O1" s="12" t="n"/>
@@ -816,30 +868,10 @@
       <c r="Y1" s="12" t="n"/>
       <c r="Z1" s="12" t="n"/>
     </row>
-    <row r="2" ht="30" customHeight="1" s="43">
-      <c r="A2" s="51" t="n"/>
-      <c r="B2" s="52" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="E2" s="51" t="n"/>
-      <c r="F2" s="62" t="n"/>
-      <c r="G2" s="62" t="n"/>
-      <c r="H2" s="63" t="n"/>
-      <c r="I2" s="54" t="n"/>
-      <c r="J2" s="64" t="inlineStr">
-        <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="K2" s="64" t="inlineStr">
-        <is>
-          <t>Amount to be released (INR) inclusive of GST</t>
-        </is>
-      </c>
-      <c r="L2" s="64" t="inlineStr">
-        <is>
-          <t>Milestone/Deliverables that will be completed  by the timeline</t>
-        </is>
-      </c>
+    <row r="2" ht="1.5" customHeight="1" s="43">
+      <c r="J2" s="37" t="n"/>
+      <c r="K2" s="37" t="n"/>
+      <c r="L2" s="37" t="n"/>
       <c r="M2" s="12" t="n"/>
       <c r="N2" s="12" t="n"/>
       <c r="O2" s="12" t="n"/>
@@ -855,46 +887,57 @@
       <c r="Y2" s="12" t="n"/>
       <c r="Z2" s="12" t="n"/>
     </row>
-    <row r="3" ht="30" customHeight="1" s="43">
-      <c r="A3" s="21" t="inlineStr">
+    <row r="3" ht="34" customHeight="1" s="43">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Sr. No.</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="58" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="58" t="inlineStr">
         <is>
           <t>Total (Rs.)</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="E3" s="58" t="inlineStr">
         <is>
           <t>S No</t>
         </is>
       </c>
-      <c r="F3" s="64" t="inlineStr">
+      <c r="F3" s="58" t="inlineStr">
         <is>
-          <t>Milestone/Deliverable</t>
+          <t>Milestone / Deliverable</t>
         </is>
       </c>
-      <c r="G3" s="65" t="inlineStr">
+      <c r="G3" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time Period </t>
+          <t>Time period</t>
         </is>
       </c>
-      <c r="H3" s="66" t="inlineStr">
+      <c r="H3" s="58" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="I3" s="54" t="n"/>
-      <c r="J3" s="67" t="n"/>
-      <c r="K3" s="67" t="n"/>
-      <c r="L3" s="67" t="n"/>
+      <c r="J3" s="58" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="K3" s="58" t="inlineStr">
+        <is>
+          <t>Amount to be released (INR)</t>
+        </is>
+      </c>
+      <c r="L3" s="58" t="inlineStr">
+        <is>
+          <t>Milestone / deliverables completed</t>
+        </is>
+      </c>
       <c r="M3" s="12" t="n"/>
       <c r="N3" s="12" t="n"/>
       <c r="O3" s="12" t="n"/>
@@ -910,46 +953,47 @@
       <c r="Y3" s="12" t="n"/>
       <c r="Z3" s="12" t="n"/>
     </row>
-    <row r="4" ht="30" customHeight="1" s="43">
-      <c r="A4" s="27" t="n">
+    <row r="4" ht="29" customHeight="1" s="43">
+      <c r="A4" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manpower </t>
+          <t>Manpower</t>
         </is>
       </c>
-      <c r="C4" s="25" t="n">
+      <c r="C4" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
+      <c r="E4" s="59" t="inlineStr">
         <is>
-          <t>Project beginning (T0)</t>
+          <t>1</t>
         </is>
       </c>
-      <c r="G4" s="66" t="inlineStr">
+      <c r="F4" s="59" t="inlineStr">
         <is>
-          <t>T0</t>
+          <t>Milestone 1: Monitor prototype</t>
         </is>
       </c>
-      <c r="H4" s="68" t="inlineStr">
+      <c r="G4" s="59" t="inlineStr">
         <is>
-          <t>Project plan, stakeholder alignment, BOM freeze</t>
+          <t>T0 + 2 months</t>
         </is>
       </c>
-      <c r="I4" s="54" t="n"/>
-      <c r="J4" s="66" t="inlineStr">
+      <c r="H4" s="59" t="inlineStr">
         <is>
-          <t>Project Start Date (T0)</t>
+          <t>M1 calibrated, score validated</t>
         </is>
       </c>
-      <c r="K4" s="69" t="n">
+      <c r="J4" s="59" t="inlineStr">
+        <is>
+          <t>Project start (T0)</t>
+        </is>
+      </c>
+      <c r="K4" s="60" t="n">
         <v>8235</v>
       </c>
-      <c r="L4" s="66" t="inlineStr">
+      <c r="L4" s="59" t="inlineStr">
         <is>
           <t>M1 monitor build and dashboard</t>
         </is>
@@ -969,46 +1013,47 @@
       <c r="Y4" s="12" t="n"/>
       <c r="Z4" s="12" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1" s="43">
-      <c r="A5" s="27" t="n">
+    <row r="5" ht="29" customHeight="1" s="43">
+      <c r="A5" s="61" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipment </t>
+          <t>Equipment (exclusive of GST)</t>
         </is>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="62" t="n">
         <v>15600</v>
       </c>
-      <c r="E5" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" s="70" t="inlineStr">
+      <c r="E5" s="61" t="inlineStr">
         <is>
-          <t>Milestone 1: Requirements and monitor prototype</t>
+          <t>2</t>
         </is>
       </c>
-      <c r="G5" s="66" t="inlineStr">
+      <c r="F5" s="61" t="inlineStr">
         <is>
-          <t>T0 + 2 months</t>
+          <t>Milestone 2: Home unit and dashboard</t>
         </is>
       </c>
-      <c r="H5" s="66" t="inlineStr">
+      <c r="G5" s="61" t="inlineStr">
         <is>
-          <t>M1 calibrated; TankScore validated; dashboard from flash</t>
+          <t>T0 + 4 months</t>
         </is>
       </c>
-      <c r="I5" s="54" t="n"/>
-      <c r="J5" s="66" t="inlineStr">
+      <c r="H5" s="61" t="inlineStr">
         <is>
-          <t>T0 + 06 months</t>
+          <t>H1 pump control, dashboard live</t>
         </is>
       </c>
-      <c r="K5" s="69" t="n">
+      <c r="J5" s="61" t="inlineStr">
+        <is>
+          <t>T0 + 6 months</t>
+        </is>
+      </c>
+      <c r="K5" s="62" t="n">
         <v>9415</v>
       </c>
-      <c r="L5" s="66" t="inlineStr">
+      <c r="L5" s="61" t="inlineStr">
         <is>
           <t>H1 home unit and C1 cleaning arm</t>
         </is>
@@ -1028,46 +1073,47 @@
       <c r="Y5" s="12" t="n"/>
       <c r="Z5" s="12" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1" s="43">
-      <c r="A6" s="27" t="n">
+    <row r="6" ht="29" customHeight="1" s="43">
+      <c r="A6" s="59" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consumables </t>
+          <t>Consumables</t>
         </is>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="70" t="inlineStr">
+      <c r="E6" s="59" t="inlineStr">
         <is>
-          <t>Milestone 2: Home unit and dashboard</t>
+          <t>3</t>
         </is>
       </c>
-      <c r="G6" s="66" t="inlineStr">
+      <c r="F6" s="59" t="inlineStr">
         <is>
-          <t>T0 + 4 months</t>
+          <t>Milestone 3: Cleaning arm</t>
         </is>
       </c>
-      <c r="H6" s="66" t="inlineStr">
+      <c r="G6" s="59" t="inlineStr">
         <is>
-          <t>H1 TFT + pump control; dashboard and session log</t>
+          <t>T0 + 8 months</t>
         </is>
       </c>
-      <c r="I6" s="54" t="n"/>
-      <c r="J6" s="66" t="inlineStr">
+      <c r="H6" s="59" t="inlineStr">
+        <is>
+          <t>C1 built, coverage measured</t>
+        </is>
+      </c>
+      <c r="J6" s="59" t="inlineStr">
         <is>
           <t>T0 + 12 months</t>
         </is>
       </c>
-      <c r="K6" s="69" t="n">
+      <c r="K6" s="60" t="n">
         <v>5937</v>
       </c>
-      <c r="L6" s="66" t="inlineStr">
+      <c r="L6" s="59" t="inlineStr">
         <is>
           <t>Field validation and evidence pack</t>
         </is>
@@ -1087,46 +1133,47 @@
       <c r="Y6" s="12" t="n"/>
       <c r="Z6" s="12" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1" s="43">
-      <c r="A7" s="27" t="n">
+    <row r="7" ht="29" customHeight="1" s="43">
+      <c r="A7" s="61" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travel </t>
+          <t>Travel</t>
         </is>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="70" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
-          <t>Milestone 3: Cleaning arm</t>
+          <t>4</t>
         </is>
       </c>
-      <c r="G7" s="66" t="inlineStr">
+      <c r="F7" s="61" t="inlineStr">
         <is>
-          <t>T0 + 8 months</t>
+          <t>Milestone 4: Field validation</t>
         </is>
       </c>
-      <c r="H7" s="66" t="inlineStr">
+      <c r="G7" s="61" t="inlineStr">
         <is>
-          <t>C1 built; three-ring cycle; coverage measured</t>
+          <t>T0 + 12 months</t>
         </is>
       </c>
-      <c r="I7" s="54" t="n"/>
-      <c r="J7" s="66" t="inlineStr">
+      <c r="H7" s="61" t="inlineStr">
+        <is>
+          <t>3 sites, 90 days, TRL 6 pack</t>
+        </is>
+      </c>
+      <c r="J7" s="63" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="K7" s="69" t="n">
+      <c r="K7" s="64" t="n">
         <v>23587</v>
       </c>
-      <c r="L7" s="66" t="inlineStr"/>
+      <c r="L7" s="63" t="inlineStr"/>
       <c r="M7" s="12" t="n"/>
       <c r="N7" s="12" t="n"/>
       <c r="O7" s="12" t="n"/>
@@ -1142,40 +1189,29 @@
       <c r="Y7" s="12" t="n"/>
       <c r="Z7" s="12" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1" s="43">
-      <c r="A8" s="27" t="n">
+    <row r="8" ht="29" customHeight="1" s="43">
+      <c r="A8" s="59" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>Miscellaneous expenses</t>
         </is>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="27" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="71" t="inlineStr">
+      <c r="E8" s="65" t="n"/>
+      <c r="F8" s="65" t="inlineStr">
         <is>
-          <t>Milestone 4: Field validation</t>
+          <t>Total</t>
         </is>
       </c>
-      <c r="G8" s="66" t="inlineStr">
-        <is>
-          <t>T0 + 12 months</t>
-        </is>
-      </c>
-      <c r="H8" s="66" t="inlineStr">
-        <is>
-          <t>Three installations, 90 days, TRL 6+ evidence</t>
-        </is>
-      </c>
-      <c r="I8" s="54" t="n"/>
-      <c r="J8" s="66" t="n"/>
-      <c r="K8" s="72" t="n"/>
-      <c r="L8" s="66" t="n"/>
+      <c r="G8" s="65" t="inlineStr"/>
+      <c r="H8" s="65" t="inlineStr"/>
+      <c r="J8" s="36" t="n"/>
+      <c r="K8" s="39" t="n"/>
+      <c r="L8" s="12" t="n"/>
       <c r="M8" s="12" t="n"/>
       <c r="N8" s="12" t="n"/>
       <c r="O8" s="12" t="n"/>
@@ -1191,34 +1227,24 @@
       <c r="Y8" s="12" t="n"/>
       <c r="Z8" s="12" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1" s="43">
-      <c r="A9" s="27" t="n">
+    <row r="9" ht="29" customHeight="1" s="43">
+      <c r="A9" s="61" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>Contingency (max 5%)</t>
         </is>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="62" t="n">
         <v>780</v>
       </c>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="66" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="G9" s="66" t="n"/>
-      <c r="H9" s="61" t="n"/>
-      <c r="I9" s="54" t="n"/>
-      <c r="J9" s="66" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="K9" s="69" t="n"/>
-      <c r="L9" s="66" t="n"/>
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="36" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="J9" s="36" t="n"/>
+      <c r="K9" s="66" t="n"/>
+      <c r="L9" s="12" t="n"/>
       <c r="M9" s="12" t="n"/>
       <c r="N9" s="12" t="n"/>
       <c r="O9" s="12" t="n"/>
@@ -1234,26 +1260,26 @@
       <c r="Y9" s="12" t="n"/>
       <c r="Z9" s="12" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1" s="43">
-      <c r="A10" s="27" t="n">
+    <row r="10" ht="29" customHeight="1" s="43">
+      <c r="A10" s="65" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="27" t="inlineStr">
+      <c r="B10" s="65" t="inlineStr">
         <is>
           <t>Sub total</t>
         </is>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="67" t="n">
         <v>16380</v>
       </c>
       <c r="E10" s="36" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="74" t="n"/>
-      <c r="H10" s="75" t="n"/>
+      <c r="F10" s="37" t="n"/>
+      <c r="G10" s="38" t="n"/>
+      <c r="H10" s="39" t="n"/>
       <c r="I10" s="12" t="n"/>
-      <c r="J10" s="76" t="n"/>
-      <c r="K10" s="76" t="n"/>
-      <c r="L10" s="76" t="n"/>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="12" t="n"/>
       <c r="M10" s="12" t="n"/>
       <c r="N10" s="12" t="n"/>
       <c r="O10" s="12" t="n"/>
@@ -1269,26 +1295,26 @@
       <c r="Y10" s="12" t="n"/>
       <c r="Z10" s="12" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1" s="43">
-      <c r="A11" s="27" t="n">
+    <row r="11" ht="29" customHeight="1" s="43">
+      <c r="A11" s="61" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="27" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overhead </t>
+          <t>Overhead (max 20%)</t>
         </is>
       </c>
-      <c r="C11" s="25" t="n">
+      <c r="C11" s="62" t="n">
         <v>3276</v>
       </c>
       <c r="E11" s="40" t="n"/>
-      <c r="F11" s="76" t="n"/>
-      <c r="G11" s="76" t="n"/>
-      <c r="H11" s="77" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="41" t="n"/>
       <c r="I11" s="12" t="n"/>
-      <c r="J11" s="76" t="n"/>
-      <c r="K11" s="76" t="n"/>
-      <c r="L11" s="76" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12" t="n"/>
       <c r="M11" s="12" t="n"/>
       <c r="N11" s="12" t="n"/>
       <c r="O11" s="12" t="n"/>
@@ -1304,26 +1330,26 @@
       <c r="Y11" s="12" t="n"/>
       <c r="Z11" s="12" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1" s="43">
-      <c r="A12" s="27" t="n">
+    <row r="12" ht="29" customHeight="1" s="43">
+      <c r="A12" s="59" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="27" t="inlineStr">
+      <c r="B12" s="59" t="inlineStr">
         <is>
           <t>Faculty fee (max 20%)</t>
         </is>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="C12" s="60" t="n">
         <v>3931</v>
       </c>
       <c r="E12" s="40" t="n"/>
-      <c r="F12" s="76" t="n"/>
-      <c r="G12" s="76" t="n"/>
-      <c r="H12" s="77" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="41" t="n"/>
       <c r="I12" s="12" t="n"/>
-      <c r="J12" s="76" t="n"/>
-      <c r="K12" s="76" t="n"/>
-      <c r="L12" s="76" t="n"/>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="12" t="n"/>
       <c r="M12" s="12" t="n"/>
       <c r="N12" s="12" t="n"/>
       <c r="O12" s="12" t="n"/>
@@ -1339,26 +1365,26 @@
       <c r="Y12" s="12" t="n"/>
       <c r="Z12" s="12" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1" s="43">
-      <c r="A13" s="27" t="n">
+    <row r="13" ht="29" customHeight="1" s="43">
+      <c r="A13" s="63" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="63" t="inlineStr">
         <is>
-          <t>Total (7+8 +9)</t>
+          <t>Total (7+8+9)</t>
         </is>
       </c>
-      <c r="C13" s="32" t="n">
+      <c r="C13" s="64" t="n">
         <v>23587</v>
       </c>
       <c r="E13" s="40" t="n"/>
-      <c r="F13" s="76" t="n"/>
-      <c r="G13" s="76" t="n"/>
-      <c r="H13" s="78" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="40" t="n"/>
       <c r="I13" s="12" t="n"/>
-      <c r="J13" s="76" t="n"/>
-      <c r="K13" s="76" t="n"/>
-      <c r="L13" s="76" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12" t="n"/>
       <c r="M13" s="12" t="n"/>
       <c r="N13" s="12" t="n"/>
       <c r="O13" s="12" t="n"/>
@@ -1374,26 +1400,26 @@
       <c r="Y13" s="12" t="n"/>
       <c r="Z13" s="12" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1" s="43">
-      <c r="A14" s="27" t="n">
+    <row r="14" ht="29" customHeight="1" s="43">
+      <c r="A14" s="59" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>GST (@18% of 10)</t>
+          <t>GST (18% of 10)</t>
         </is>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="60" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="12" t="n"/>
-      <c r="F14" s="76" t="n"/>
-      <c r="G14" s="76" t="n"/>
-      <c r="H14" s="76" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
       <c r="I14" s="12" t="n"/>
-      <c r="J14" s="76" t="n"/>
-      <c r="K14" s="76" t="n"/>
-      <c r="L14" s="76" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="12" t="n"/>
       <c r="M14" s="12" t="n"/>
       <c r="N14" s="12" t="n"/>
       <c r="O14" s="12" t="n"/>
@@ -1409,27 +1435,26 @@
       <c r="Y14" s="12" t="n"/>
       <c r="Z14" s="12" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1" s="43">
-      <c r="A15" s="27" t="n">
+    <row r="15" ht="29" customHeight="1" s="43">
+      <c r="A15" s="63" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="63" t="inlineStr">
         <is>
-          <t>Grant Total (10+11)</t>
+          <t>Grand total (10+11)</t>
         </is>
       </c>
-      <c r="C15" s="32" t="n">
+      <c r="C15" s="64" t="n">
         <v>23587</v>
       </c>
-      <c r="D15" s="56" t="n"/>
       <c r="E15" s="12" t="n"/>
-      <c r="F15" s="76" t="n"/>
-      <c r="G15" s="76" t="n"/>
-      <c r="H15" s="76" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
       <c r="I15" s="12" t="n"/>
-      <c r="J15" s="76" t="n"/>
-      <c r="K15" s="76" t="n"/>
-      <c r="L15" s="76" t="n"/>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="12" t="n"/>
       <c r="M15" s="12" t="n"/>
       <c r="N15" s="12" t="n"/>
       <c r="O15" s="12" t="n"/>
@@ -29026,20 +29051,14 @@
       <c r="Z1000" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="I1:I9"/>
+  <mergeCells count="3">
     <mergeCell ref="J1:L1"/>
-    <mergeCell ref="D1:D15"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="E1:H2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="E1:H1"/>
   </mergeCells>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.35" right="0.35" top="0.4" bottom="0.4" header="0" footer="0"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -29049,26 +29068,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z997"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="43" min="1" max="2"/>
-    <col width="25.43" customWidth="1" style="43" min="3" max="3"/>
-    <col width="17.71" customWidth="1" style="43" min="4" max="4"/>
+    <col width="6" customWidth="1" style="43" min="2" max="2"/>
+    <col width="44" customWidth="1" style="43" min="3" max="3"/>
+    <col width="24" customWidth="1" style="43" min="4" max="4"/>
     <col width="17.86" customWidth="1" style="43" min="5" max="5"/>
     <col width="17.14" customWidth="1" style="43" min="6" max="6"/>
     <col width="20.43" customWidth="1" style="43" min="7" max="7"/>
     <col width="8.710000000000001" customWidth="1" style="43" min="8" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="43">
+    <row r="1" ht="14.25" customHeight="1" s="43">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="79" t="n"/>
-      <c r="C1" s="79" t="n"/>
-      <c r="D1" s="79" t="n"/>
-      <c r="E1" s="79" t="n"/>
-      <c r="F1" s="79" t="n"/>
-      <c r="G1" s="79" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
@@ -29089,19 +29109,17 @@
       <c r="Y1" s="1" t="n"/>
       <c r="Z1" s="1" t="n"/>
     </row>
-    <row r="2" ht="26" customHeight="1" s="43">
+    <row r="2" ht="24" customHeight="1" s="43">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="79" t="n"/>
-      <c r="C2" s="79" t="n"/>
-      <c r="D2" s="79" t="n"/>
-      <c r="E2" s="79" t="n"/>
-      <c r="F2" s="79" t="n"/>
-      <c r="G2" s="79" t="n"/>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="B2" s="68" t="inlineStr">
         <is>
-          <t>Grant total: INR 23,587</t>
+          <t>Milestone Expenditure Sheet</t>
         </is>
       </c>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
@@ -29121,38 +29139,17 @@
       <c r="Y2" s="1" t="n"/>
       <c r="Z2" s="1" t="n"/>
     </row>
-    <row r="3" ht="26" customHeight="1" s="43">
+    <row r="3">
       <c r="A3" s="1" t="n"/>
-      <c r="B3" s="80" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
-          <t>Milestone Expenditure Sheet</t>
+          <t>Grant total: INR 23,587</t>
         </is>
       </c>
-      <c r="C3" s="60" t="n"/>
-      <c r="D3" s="61" t="n"/>
-      <c r="E3" s="80" t="inlineStr">
-        <is>
-          <t>Tranche 1
-8,235</t>
-        </is>
-      </c>
-      <c r="F3" s="80" t="inlineStr">
-        <is>
-          <t>Tranche 2
-9,415</t>
-        </is>
-      </c>
-      <c r="G3" s="80" t="inlineStr">
-        <is>
-          <t>Tranche 3
-5,937</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Add columns </t>
-        </is>
-      </c>
+      <c r="E3" s="70" t="n"/>
+      <c r="F3" s="70" t="n"/>
+      <c r="G3" s="70" t="n"/>
+      <c r="H3" s="1" t="n"/>
       <c r="I3" s="1" t="n"/>
       <c r="J3" s="1" t="n"/>
       <c r="K3" s="1" t="n"/>
@@ -29172,42 +29169,26 @@
       <c r="Y3" s="1" t="n"/>
       <c r="Z3" s="1" t="n"/>
     </row>
-    <row r="4" ht="26" customHeight="1" s="43">
+    <row r="4" ht="14.25" customHeight="1" s="43">
       <c r="A4" s="1" t="n"/>
-      <c r="B4" s="80" t="inlineStr">
+      <c r="B4" s="58" t="inlineStr">
         <is>
-          <t>Sr.No.</t>
+          <t>Sr. No.</t>
         </is>
       </c>
-      <c r="C4" s="80" t="inlineStr">
+      <c r="C4" s="58" t="inlineStr">
         <is>
-          <t>Expenditure Heads</t>
+          <t>Expenditure heads</t>
         </is>
       </c>
-      <c r="D4" s="80" t="inlineStr">
+      <c r="D4" s="58" t="inlineStr">
         <is>
-          <t>Total Funding
-Amount</t>
+          <t>Total funding (INR)</t>
         </is>
       </c>
-      <c r="E4" s="80" t="inlineStr">
-        <is>
-          <t>Budgeted
-Amount</t>
-        </is>
-      </c>
-      <c r="F4" s="80" t="inlineStr">
-        <is>
-          <t>Budgeted
-Amount</t>
-        </is>
-      </c>
-      <c r="G4" s="80" t="inlineStr">
-        <is>
-          <t>Budgeted
-Amount</t>
-        </is>
-      </c>
+      <c r="E4" s="70" t="n"/>
+      <c r="F4" s="70" t="n"/>
+      <c r="G4" s="70" t="n"/>
       <c r="H4" s="1" t="n"/>
       <c r="I4" s="1" t="n"/>
       <c r="J4" s="1" t="n"/>
@@ -29228,22 +29209,22 @@
       <c r="Y4" s="1" t="n"/>
       <c r="Z4" s="1" t="n"/>
     </row>
-    <row r="5" ht="26" customHeight="1" s="43">
+    <row r="5" ht="22" customHeight="1" s="43">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="81" t="n">
+      <c r="B5" s="71" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="66" t="inlineStr">
+      <c r="C5" s="61" t="inlineStr">
         <is>
           <t>Manpower</t>
         </is>
       </c>
-      <c r="D5" s="82" t="n">
+      <c r="D5" s="72" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="81" t="n"/>
-      <c r="F5" s="81" t="n"/>
-      <c r="G5" s="81" t="n"/>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
       <c r="H5" s="1" t="n"/>
       <c r="I5" s="1" t="n"/>
       <c r="J5" s="1" t="n"/>
@@ -29264,22 +29245,22 @@
       <c r="Y5" s="1" t="n"/>
       <c r="Z5" s="1" t="n"/>
     </row>
-    <row r="6" ht="26" customHeight="1" s="43">
+    <row r="6" ht="22" customHeight="1" s="43">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="81" t="n">
+      <c r="B6" s="73" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="66" t="inlineStr">
+      <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>Equipment (Exclusive of GST)</t>
+          <t>Equipment (exclusive of GST)</t>
         </is>
       </c>
-      <c r="D6" s="82" t="n">
+      <c r="D6" s="74" t="n">
         <v>15600</v>
       </c>
-      <c r="E6" s="81" t="n"/>
-      <c r="F6" s="81" t="n"/>
-      <c r="G6" s="81" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="n"/>
@@ -29300,22 +29281,22 @@
       <c r="Y6" s="1" t="n"/>
       <c r="Z6" s="1" t="n"/>
     </row>
-    <row r="7" ht="26" customHeight="1" s="43">
+    <row r="7" ht="22" customHeight="1" s="43">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="81" t="n">
+      <c r="B7" s="71" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="66" t="inlineStr">
+      <c r="C7" s="61" t="inlineStr">
         <is>
-          <t>Contingency (max 5%)</t>
+          <t>Consumables</t>
         </is>
       </c>
-      <c r="D7" s="82" t="n">
-        <v>780</v>
+      <c r="D7" s="72" t="n">
+        <v>0</v>
       </c>
-      <c r="E7" s="81" t="n"/>
-      <c r="F7" s="81" t="n"/>
-      <c r="G7" s="81" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
       <c r="J7" s="1" t="n"/>
@@ -29336,22 +29317,22 @@
       <c r="Y7" s="1" t="n"/>
       <c r="Z7" s="1" t="n"/>
     </row>
-    <row r="8" ht="26" customHeight="1" s="43">
+    <row r="8" ht="22" customHeight="1" s="43">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="81" t="n">
+      <c r="B8" s="73" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="66" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr">
         <is>
-          <t>Sub total</t>
+          <t>Travel</t>
         </is>
       </c>
-      <c r="D8" s="82" t="n">
-        <v>16380</v>
+      <c r="D8" s="74" t="n">
+        <v>0</v>
       </c>
-      <c r="E8" s="81" t="n"/>
-      <c r="F8" s="81" t="n"/>
-      <c r="G8" s="81" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
       <c r="J8" s="1" t="n"/>
@@ -29372,22 +29353,22 @@
       <c r="Y8" s="1" t="n"/>
       <c r="Z8" s="1" t="n"/>
     </row>
-    <row r="9" ht="26" customHeight="1" s="43">
+    <row r="9" ht="22" customHeight="1" s="43">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="81" t="n">
+      <c r="B9" s="71" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="64" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr">
         <is>
-          <t>Overhead (max 20%)</t>
+          <t>Miscellaneous expenses</t>
         </is>
       </c>
-      <c r="D9" s="82" t="n">
-        <v>3276</v>
+      <c r="D9" s="72" t="n">
+        <v>0</v>
       </c>
-      <c r="E9" s="81" t="n"/>
-      <c r="F9" s="81" t="n"/>
-      <c r="G9" s="81" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
       <c r="J9" s="1" t="n"/>
@@ -29408,22 +29389,22 @@
       <c r="Y9" s="1" t="n"/>
       <c r="Z9" s="1" t="n"/>
     </row>
-    <row r="10" ht="26" customHeight="1" s="43">
+    <row r="10" ht="22" customHeight="1" s="43">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="81" t="n">
+      <c r="B10" s="73" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="66" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr">
         <is>
-          <t>Faculty Fee (max 20%)</t>
+          <t>Contingency (max 5%)</t>
         </is>
       </c>
-      <c r="D10" s="82" t="n">
-        <v>3931</v>
+      <c r="D10" s="74" t="n">
+        <v>780</v>
       </c>
-      <c r="E10" s="81" t="n"/>
-      <c r="F10" s="81" t="n"/>
-      <c r="G10" s="81" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
       <c r="J10" s="1" t="n"/>
@@ -29444,22 +29425,22 @@
       <c r="Y10" s="1" t="n"/>
       <c r="Z10" s="1" t="n"/>
     </row>
-    <row r="11" ht="26" customHeight="1" s="43">
+    <row r="11" ht="22" customHeight="1" s="43">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="81" t="n">
+      <c r="B11" s="75" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="64" t="inlineStr">
+      <c r="C11" s="63" t="inlineStr">
         <is>
-          <t>Total (7+8+9)</t>
+          <t>Sub total</t>
         </is>
       </c>
-      <c r="D11" s="82" t="n">
-        <v>23587</v>
+      <c r="D11" s="76" t="n">
+        <v>16380</v>
       </c>
-      <c r="E11" s="81" t="n"/>
-      <c r="F11" s="81" t="n"/>
-      <c r="G11" s="81" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="1" t="n"/>
@@ -29480,14 +29461,22 @@
       <c r="Y11" s="1" t="n"/>
       <c r="Z11" s="1" t="n"/>
     </row>
-    <row r="12" ht="26" customHeight="1" s="43">
+    <row r="12" ht="22" customHeight="1" s="43">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="81" t="n"/>
-      <c r="C12" s="81" t="n"/>
-      <c r="D12" s="81" t="n"/>
-      <c r="E12" s="81" t="n"/>
-      <c r="F12" s="81" t="n"/>
-      <c r="G12" s="81" t="n"/>
+      <c r="B12" s="73" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>Overhead (max 20%)</t>
+        </is>
+      </c>
+      <c r="D12" s="74" t="n">
+        <v>3276</v>
+      </c>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
       <c r="J12" s="1" t="n"/>
@@ -29508,18 +29497,22 @@
       <c r="Y12" s="1" t="n"/>
       <c r="Z12" s="1" t="n"/>
     </row>
-    <row r="13" ht="20" customHeight="1" s="43">
+    <row r="13" ht="22" customHeight="1" s="43">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="83" t="inlineStr">
+      <c r="B13" s="71" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
         <is>
-          <t>80% of the tranche fund should be utilized before claiming for the next tranche.</t>
+          <t>Faculty fee (max 20%)</t>
         </is>
       </c>
-      <c r="C13" s="60" t="n"/>
-      <c r="D13" s="60" t="n"/>
-      <c r="E13" s="60" t="n"/>
-      <c r="F13" s="61" t="n"/>
-      <c r="G13" s="81" t="n"/>
+      <c r="D13" s="72" t="n">
+        <v>3931</v>
+      </c>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="n"/>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
       <c r="J13" s="1" t="n"/>
@@ -29540,14 +29533,22 @@
       <c r="Y13" s="1" t="n"/>
       <c r="Z13" s="1" t="n"/>
     </row>
-    <row r="14" ht="26" customHeight="1" s="43">
+    <row r="14" ht="22" customHeight="1" s="43">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="79" t="n"/>
-      <c r="C14" s="79" t="n"/>
-      <c r="D14" s="79" t="n"/>
-      <c r="E14" s="79" t="n"/>
-      <c r="F14" s="79" t="n"/>
-      <c r="G14" s="79" t="n"/>
+      <c r="B14" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="65" t="inlineStr">
+        <is>
+          <t>Total (7+8+9)</t>
+        </is>
+      </c>
+      <c r="D14" s="78" t="n">
+        <v>23587</v>
+      </c>
+      <c r="E14" s="1" t="n"/>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="n"/>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
       <c r="J14" s="1" t="n"/>
@@ -29568,14 +29569,22 @@
       <c r="Y14" s="1" t="n"/>
       <c r="Z14" s="1" t="n"/>
     </row>
-    <row r="15" ht="26" customHeight="1" s="43">
+    <row r="15" ht="22" customHeight="1" s="43">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="79" t="n"/>
-      <c r="C15" s="79" t="n"/>
-      <c r="D15" s="79" t="n"/>
-      <c r="E15" s="79" t="n"/>
-      <c r="F15" s="79" t="n"/>
-      <c r="G15" s="79" t="n"/>
+      <c r="B15" s="71" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>GST (18% of 10)</t>
+        </is>
+      </c>
+      <c r="D15" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="n"/>
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="n"/>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
       <c r="J15" s="1" t="n"/>
@@ -29596,14 +29605,22 @@
       <c r="Y15" s="1" t="n"/>
       <c r="Z15" s="1" t="n"/>
     </row>
-    <row r="16" ht="26" customHeight="1" s="43">
+    <row r="16" ht="22" customHeight="1" s="43">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="79" t="n"/>
-      <c r="C16" s="79" t="n"/>
-      <c r="D16" s="79" t="n"/>
+      <c r="B16" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" s="65" t="inlineStr">
+        <is>
+          <t>Grand total (10+11)</t>
+        </is>
+      </c>
+      <c r="D16" s="78" t="n">
+        <v>23587</v>
+      </c>
       <c r="E16" s="79" t="n"/>
       <c r="F16" s="79" t="n"/>
-      <c r="G16" s="79" t="n"/>
+      <c r="G16" s="1" t="n"/>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
@@ -29624,14 +29641,14 @@
       <c r="Y16" s="1" t="n"/>
       <c r="Z16" s="1" t="n"/>
     </row>
-    <row r="17" ht="26" customHeight="1" s="43">
+    <row r="17" ht="14.25" customHeight="1" s="43">
       <c r="A17" s="1" t="n"/>
       <c r="B17" s="79" t="n"/>
       <c r="C17" s="79" t="n"/>
       <c r="D17" s="79" t="n"/>
       <c r="E17" s="79" t="n"/>
       <c r="F17" s="79" t="n"/>
-      <c r="G17" s="79" t="n"/>
+      <c r="G17" s="1" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
       <c r="J17" s="1" t="n"/>
@@ -29652,13 +29669,13 @@
       <c r="Y17" s="1" t="n"/>
       <c r="Z17" s="1" t="n"/>
     </row>
-    <row r="18" ht="14.25" customHeight="1" s="43">
+    <row r="18" ht="30" customHeight="1" s="43">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
+      <c r="B18" s="80" t="inlineStr">
+        <is>
+          <t>80 percent of each tranche is spent before the next is claimed. Tranche amounts are set out on the Milestones sheet.</t>
+        </is>
+      </c>
       <c r="G18" s="1" t="n"/>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
@@ -57092,18 +57109,154 @@
       <c r="Y997" s="1" t="n"/>
       <c r="Z997" s="1" t="n"/>
     </row>
-    <row r="998" ht="14.25" customHeight="1" s="43"/>
-    <row r="999" ht="14.25" customHeight="1" s="43"/>
-    <row r="1000" ht="14.25" customHeight="1" s="43"/>
-    <row r="1001" ht="14.25" customHeight="1" s="43"/>
-    <row r="1002" ht="14.25" customHeight="1" s="43"/>
+    <row r="998" ht="14.25" customHeight="1" s="43">
+      <c r="A998" s="1" t="n"/>
+      <c r="B998" s="1" t="n"/>
+      <c r="C998" s="1" t="n"/>
+      <c r="D998" s="1" t="n"/>
+      <c r="E998" s="1" t="n"/>
+      <c r="F998" s="1" t="n"/>
+      <c r="G998" s="1" t="n"/>
+      <c r="H998" s="1" t="n"/>
+      <c r="I998" s="1" t="n"/>
+      <c r="J998" s="1" t="n"/>
+      <c r="K998" s="1" t="n"/>
+      <c r="L998" s="1" t="n"/>
+      <c r="M998" s="1" t="n"/>
+      <c r="N998" s="1" t="n"/>
+      <c r="O998" s="1" t="n"/>
+      <c r="P998" s="1" t="n"/>
+      <c r="Q998" s="1" t="n"/>
+      <c r="R998" s="1" t="n"/>
+      <c r="S998" s="1" t="n"/>
+      <c r="T998" s="1" t="n"/>
+      <c r="U998" s="1" t="n"/>
+      <c r="V998" s="1" t="n"/>
+      <c r="W998" s="1" t="n"/>
+      <c r="X998" s="1" t="n"/>
+      <c r="Y998" s="1" t="n"/>
+      <c r="Z998" s="1" t="n"/>
+    </row>
+    <row r="999" ht="14.25" customHeight="1" s="43">
+      <c r="A999" s="1" t="n"/>
+      <c r="B999" s="1" t="n"/>
+      <c r="C999" s="1" t="n"/>
+      <c r="D999" s="1" t="n"/>
+      <c r="E999" s="1" t="n"/>
+      <c r="F999" s="1" t="n"/>
+      <c r="G999" s="1" t="n"/>
+      <c r="H999" s="1" t="n"/>
+      <c r="I999" s="1" t="n"/>
+      <c r="J999" s="1" t="n"/>
+      <c r="K999" s="1" t="n"/>
+      <c r="L999" s="1" t="n"/>
+      <c r="M999" s="1" t="n"/>
+      <c r="N999" s="1" t="n"/>
+      <c r="O999" s="1" t="n"/>
+      <c r="P999" s="1" t="n"/>
+      <c r="Q999" s="1" t="n"/>
+      <c r="R999" s="1" t="n"/>
+      <c r="S999" s="1" t="n"/>
+      <c r="T999" s="1" t="n"/>
+      <c r="U999" s="1" t="n"/>
+      <c r="V999" s="1" t="n"/>
+      <c r="W999" s="1" t="n"/>
+      <c r="X999" s="1" t="n"/>
+      <c r="Y999" s="1" t="n"/>
+      <c r="Z999" s="1" t="n"/>
+    </row>
+    <row r="1000" ht="14.25" customHeight="1" s="43">
+      <c r="A1000" s="1" t="n"/>
+      <c r="B1000" s="1" t="n"/>
+      <c r="C1000" s="1" t="n"/>
+      <c r="D1000" s="1" t="n"/>
+      <c r="E1000" s="1" t="n"/>
+      <c r="F1000" s="1" t="n"/>
+      <c r="G1000" s="1" t="n"/>
+      <c r="H1000" s="1" t="n"/>
+      <c r="I1000" s="1" t="n"/>
+      <c r="J1000" s="1" t="n"/>
+      <c r="K1000" s="1" t="n"/>
+      <c r="L1000" s="1" t="n"/>
+      <c r="M1000" s="1" t="n"/>
+      <c r="N1000" s="1" t="n"/>
+      <c r="O1000" s="1" t="n"/>
+      <c r="P1000" s="1" t="n"/>
+      <c r="Q1000" s="1" t="n"/>
+      <c r="R1000" s="1" t="n"/>
+      <c r="S1000" s="1" t="n"/>
+      <c r="T1000" s="1" t="n"/>
+      <c r="U1000" s="1" t="n"/>
+      <c r="V1000" s="1" t="n"/>
+      <c r="W1000" s="1" t="n"/>
+      <c r="X1000" s="1" t="n"/>
+      <c r="Y1000" s="1" t="n"/>
+      <c r="Z1000" s="1" t="n"/>
+    </row>
+    <row r="1001" ht="14.25" customHeight="1" s="43">
+      <c r="A1001" s="1" t="n"/>
+      <c r="B1001" s="1" t="n"/>
+      <c r="C1001" s="1" t="n"/>
+      <c r="D1001" s="1" t="n"/>
+      <c r="E1001" s="1" t="n"/>
+      <c r="F1001" s="1" t="n"/>
+      <c r="G1001" s="1" t="n"/>
+      <c r="H1001" s="1" t="n"/>
+      <c r="I1001" s="1" t="n"/>
+      <c r="J1001" s="1" t="n"/>
+      <c r="K1001" s="1" t="n"/>
+      <c r="L1001" s="1" t="n"/>
+      <c r="M1001" s="1" t="n"/>
+      <c r="N1001" s="1" t="n"/>
+      <c r="O1001" s="1" t="n"/>
+      <c r="P1001" s="1" t="n"/>
+      <c r="Q1001" s="1" t="n"/>
+      <c r="R1001" s="1" t="n"/>
+      <c r="S1001" s="1" t="n"/>
+      <c r="T1001" s="1" t="n"/>
+      <c r="U1001" s="1" t="n"/>
+      <c r="V1001" s="1" t="n"/>
+      <c r="W1001" s="1" t="n"/>
+      <c r="X1001" s="1" t="n"/>
+      <c r="Y1001" s="1" t="n"/>
+      <c r="Z1001" s="1" t="n"/>
+    </row>
+    <row r="1002" ht="14.25" customHeight="1" s="43">
+      <c r="A1002" s="1" t="n"/>
+      <c r="B1002" s="1" t="n"/>
+      <c r="C1002" s="1" t="n"/>
+      <c r="D1002" s="1" t="n"/>
+      <c r="E1002" s="1" t="n"/>
+      <c r="F1002" s="1" t="n"/>
+      <c r="G1002" s="1" t="n"/>
+      <c r="H1002" s="1" t="n"/>
+      <c r="I1002" s="1" t="n"/>
+      <c r="J1002" s="1" t="n"/>
+      <c r="K1002" s="1" t="n"/>
+      <c r="L1002" s="1" t="n"/>
+      <c r="M1002" s="1" t="n"/>
+      <c r="N1002" s="1" t="n"/>
+      <c r="O1002" s="1" t="n"/>
+      <c r="P1002" s="1" t="n"/>
+      <c r="Q1002" s="1" t="n"/>
+      <c r="R1002" s="1" t="n"/>
+      <c r="S1002" s="1" t="n"/>
+      <c r="T1002" s="1" t="n"/>
+      <c r="U1002" s="1" t="n"/>
+      <c r="V1002" s="1" t="n"/>
+      <c r="W1002" s="1" t="n"/>
+      <c r="X1002" s="1" t="n"/>
+      <c r="Y1002" s="1" t="n"/>
+      <c r="Z1002" s="1" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="B18:D18"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(office): make the grant a commercialisation request, not a parts bill
TDP 11 funds up to INR 50 lakh over 12 months for TRL 6+ projects that are ready to commercialise. The previous ask was INR 23,587, which is the prototype's parts cost and was already spent, so it read as a reimbursement request and contradicted the TRL 6 entry rule.

The request is now INR 42,33,600: two engineers, tooling, twenty pilot units, certification, a patent and twelve field installations. The prototype spend is shown as prior investment, and the milestones end at a sale rather than a demonstration.

The proposal gains a commercialisation section with the buyer, price target, market base and route to revenue. The workbook now splits every head across the three tranches, and the PI affiliation is corrected to Sree Buddha College of Engineering with Nuke Labs as the industry partner.
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -8,7 +8,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Milestones'!$A$1:$L$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$D$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$G$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##,##0"/>
+  </numFmts>
   <fonts count="17">
     <font>
       <name val="Calibri"/>
@@ -344,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -479,19 +481,19 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -500,7 +502,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -509,31 +511,28 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -963,7 +962,7 @@
         </is>
       </c>
       <c r="C4" s="60" t="n">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="E4" s="59" t="inlineStr">
         <is>
@@ -972,17 +971,17 @@
       </c>
       <c r="F4" s="59" t="inlineStr">
         <is>
-          <t>Milestone 1: Monitor prototype</t>
+          <t>Milestone 1: Design freeze and tooling</t>
         </is>
       </c>
       <c r="G4" s="59" t="inlineStr">
         <is>
-          <t>T0 + 2 months</t>
+          <t>T0 + 3 months</t>
         </is>
       </c>
       <c r="H4" s="59" t="inlineStr">
         <is>
-          <t>M1 calibrated, score validated</t>
+          <t>Moulds ordered, 5 pilot sets built</t>
         </is>
       </c>
       <c r="J4" s="59" t="inlineStr">
@@ -991,11 +990,11 @@
         </is>
       </c>
       <c r="K4" s="60" t="n">
-        <v>8235</v>
+        <v>1533168</v>
       </c>
       <c r="L4" s="59" t="inlineStr">
         <is>
-          <t>M1 monitor build and dashboard</t>
+          <t>Design freeze, tooling, first pilot sets</t>
         </is>
       </c>
       <c r="M4" s="12" t="n"/>
@@ -1023,7 +1022,7 @@
         </is>
       </c>
       <c r="C5" s="62" t="n">
-        <v>15600</v>
+        <v>600000</v>
       </c>
       <c r="E5" s="61" t="inlineStr">
         <is>
@@ -1032,17 +1031,17 @@
       </c>
       <c r="F5" s="61" t="inlineStr">
         <is>
-          <t>Milestone 2: Home unit and dashboard</t>
+          <t>Milestone 2: Pilot build and lab qualification</t>
         </is>
       </c>
       <c r="G5" s="61" t="inlineStr">
         <is>
-          <t>T0 + 4 months</t>
+          <t>T0 + 6 months</t>
         </is>
       </c>
       <c r="H5" s="61" t="inlineStr">
         <is>
-          <t>H1 pump control, dashboard live</t>
+          <t>20 sets, IP68 and EMC passed</t>
         </is>
       </c>
       <c r="J5" s="61" t="inlineStr">
@@ -1051,11 +1050,11 @@
         </is>
       </c>
       <c r="K5" s="62" t="n">
-        <v>9415</v>
+        <v>1684368</v>
       </c>
       <c r="L5" s="61" t="inlineStr">
         <is>
-          <t>H1 home unit and C1 cleaning arm</t>
+          <t>Pilot build, certification, field deployment</t>
         </is>
       </c>
       <c r="M5" s="12" t="n"/>
@@ -1083,7 +1082,7 @@
         </is>
       </c>
       <c r="C6" s="60" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="E6" s="59" t="inlineStr">
         <is>
@@ -1092,17 +1091,17 @@
       </c>
       <c r="F6" s="59" t="inlineStr">
         <is>
-          <t>Milestone 3: Cleaning arm</t>
+          <t>Milestone 3: Field deployment</t>
         </is>
       </c>
       <c r="G6" s="59" t="inlineStr">
         <is>
-          <t>T0 + 8 months</t>
+          <t>T0 + 9 months</t>
         </is>
       </c>
       <c r="H6" s="59" t="inlineStr">
         <is>
-          <t>C1 built, coverage measured</t>
+          <t>12 sites, 60 days of operation</t>
         </is>
       </c>
       <c r="J6" s="59" t="inlineStr">
@@ -1111,11 +1110,11 @@
         </is>
       </c>
       <c r="K6" s="60" t="n">
-        <v>5937</v>
+        <v>1016064</v>
       </c>
       <c r="L6" s="59" t="inlineStr">
         <is>
-          <t>Field validation and evidence pack</t>
+          <t>Validation, IP filing, commercial launch</t>
         </is>
       </c>
       <c r="M6" s="12" t="n"/>
@@ -1143,7 +1142,7 @@
         </is>
       </c>
       <c r="C7" s="62" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="E7" s="61" t="inlineStr">
         <is>
@@ -1152,7 +1151,7 @@
       </c>
       <c r="F7" s="61" t="inlineStr">
         <is>
-          <t>Milestone 4: Field validation</t>
+          <t>Milestone 4: Commercial readiness</t>
         </is>
       </c>
       <c r="G7" s="61" t="inlineStr">
@@ -1162,7 +1161,7 @@
       </c>
       <c r="H7" s="61" t="inlineStr">
         <is>
-          <t>3 sites, 90 days, TRL 6 pack</t>
+          <t>3 paying pilots, TRL 8 pack</t>
         </is>
       </c>
       <c r="J7" s="63" t="inlineStr">
@@ -1171,7 +1170,7 @@
         </is>
       </c>
       <c r="K7" s="64" t="n">
-        <v>23587</v>
+        <v>4233600</v>
       </c>
       <c r="L7" s="63" t="inlineStr"/>
       <c r="M7" s="12" t="n"/>
@@ -1199,7 +1198,7 @@
         </is>
       </c>
       <c r="C8" s="60" t="n">
-        <v>0</v>
+        <v>440000</v>
       </c>
       <c r="E8" s="65" t="n"/>
       <c r="F8" s="65" t="inlineStr">
@@ -1237,7 +1236,7 @@
         </is>
       </c>
       <c r="C9" s="62" t="n">
-        <v>780</v>
+        <v>140000</v>
       </c>
       <c r="E9" s="36" t="n"/>
       <c r="F9" s="36" t="n"/>
@@ -1270,7 +1269,7 @@
         </is>
       </c>
       <c r="C10" s="67" t="n">
-        <v>16380</v>
+        <v>2940000</v>
       </c>
       <c r="E10" s="36" t="n"/>
       <c r="F10" s="37" t="n"/>
@@ -1305,7 +1304,7 @@
         </is>
       </c>
       <c r="C11" s="62" t="n">
-        <v>3276</v>
+        <v>588000</v>
       </c>
       <c r="E11" s="40" t="n"/>
       <c r="F11" s="12" t="n"/>
@@ -1340,7 +1339,7 @@
         </is>
       </c>
       <c r="C12" s="60" t="n">
-        <v>3931</v>
+        <v>705600</v>
       </c>
       <c r="E12" s="40" t="n"/>
       <c r="F12" s="12" t="n"/>
@@ -1375,7 +1374,7 @@
         </is>
       </c>
       <c r="C13" s="64" t="n">
-        <v>23587</v>
+        <v>4233600</v>
       </c>
       <c r="E13" s="40" t="n"/>
       <c r="F13" s="12" t="n"/>
@@ -1445,7 +1444,7 @@
         </is>
       </c>
       <c r="C15" s="64" t="n">
-        <v>23587</v>
+        <v>4233600</v>
       </c>
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="12" t="n"/>
@@ -29073,11 +29072,11 @@
   <cols>
     <col width="8.710000000000001" customWidth="1" style="43" min="1" max="2"/>
     <col width="6" customWidth="1" style="43" min="2" max="2"/>
-    <col width="44" customWidth="1" style="43" min="3" max="3"/>
-    <col width="24" customWidth="1" style="43" min="4" max="4"/>
-    <col width="17.86" customWidth="1" style="43" min="5" max="5"/>
-    <col width="17.14" customWidth="1" style="43" min="6" max="6"/>
-    <col width="20.43" customWidth="1" style="43" min="7" max="7"/>
+    <col width="40" customWidth="1" style="43" min="3" max="3"/>
+    <col width="17" customWidth="1" style="43" min="4" max="4"/>
+    <col width="17" customWidth="1" style="43" min="5" max="5"/>
+    <col width="17" customWidth="1" style="43" min="6" max="6"/>
+    <col width="17" customWidth="1" style="43" min="7" max="7"/>
     <col width="8.710000000000001" customWidth="1" style="43" min="8" max="26"/>
   </cols>
   <sheetData>
@@ -29116,9 +29115,6 @@
           <t>Milestone Expenditure Sheet</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
       <c r="H2" s="1" t="n"/>
       <c r="I2" s="1" t="n"/>
       <c r="J2" s="1" t="n"/>
@@ -29143,12 +29139,9 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="69" t="inlineStr">
         <is>
-          <t>Grant total: INR 23,587</t>
+          <t>Grant total: INR 42,33,600</t>
         </is>
       </c>
-      <c r="E3" s="70" t="n"/>
-      <c r="F3" s="70" t="n"/>
-      <c r="G3" s="70" t="n"/>
       <c r="H3" s="1" t="n"/>
       <c r="I3" s="1" t="n"/>
       <c r="J3" s="1" t="n"/>
@@ -29183,12 +29176,24 @@
       </c>
       <c r="D4" s="58" t="inlineStr">
         <is>
-          <t>Total funding (INR)</t>
+          <t>Tranche 1 (T0)</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="70" t="n"/>
-      <c r="G4" s="70" t="n"/>
+      <c r="E4" s="58" t="inlineStr">
+        <is>
+          <t>Tranche 2 (T0 + 6)</t>
+        </is>
+      </c>
+      <c r="F4" s="58" t="inlineStr">
+        <is>
+          <t>Tranche 3 (T0 + 12)</t>
+        </is>
+      </c>
+      <c r="G4" s="58" t="inlineStr">
+        <is>
+          <t>Total (INR)</t>
+        </is>
+      </c>
       <c r="H4" s="1" t="n"/>
       <c r="I4" s="1" t="n"/>
       <c r="J4" s="1" t="n"/>
@@ -29211,7 +29216,7 @@
     </row>
     <row r="5" ht="22" customHeight="1" s="43">
       <c r="A5" s="1" t="n"/>
-      <c r="B5" s="71" t="n">
+      <c r="B5" s="70" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="61" t="inlineStr">
@@ -29219,12 +29224,18 @@
           <t>Manpower</t>
         </is>
       </c>
-      <c r="D5" s="72" t="n">
-        <v>0</v>
+      <c r="D5" s="71" t="n">
+        <v>360000</v>
       </c>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="1" t="n"/>
+      <c r="E5" s="71" t="n">
+        <v>480000</v>
+      </c>
+      <c r="F5" s="71" t="n">
+        <v>360000</v>
+      </c>
+      <c r="G5" s="71" t="n">
+        <v>1200000</v>
+      </c>
       <c r="H5" s="1" t="n"/>
       <c r="I5" s="1" t="n"/>
       <c r="J5" s="1" t="n"/>
@@ -29247,7 +29258,7 @@
     </row>
     <row r="6" ht="22" customHeight="1" s="43">
       <c r="A6" s="1" t="n"/>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="72" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="59" t="inlineStr">
@@ -29255,12 +29266,18 @@
           <t>Equipment (exclusive of GST)</t>
         </is>
       </c>
-      <c r="D6" s="74" t="n">
-        <v>15600</v>
+      <c r="D6" s="73" t="n">
+        <v>360000</v>
       </c>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
+      <c r="E6" s="73" t="n">
+        <v>240000</v>
+      </c>
+      <c r="F6" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="73" t="n">
+        <v>600000</v>
+      </c>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
       <c r="J6" s="1" t="n"/>
@@ -29283,7 +29300,7 @@
     </row>
     <row r="7" ht="22" customHeight="1" s="43">
       <c r="A7" s="1" t="n"/>
-      <c r="B7" s="71" t="n">
+      <c r="B7" s="70" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="61" t="inlineStr">
@@ -29291,12 +29308,18 @@
           <t>Consumables</t>
         </is>
       </c>
-      <c r="D7" s="72" t="n">
-        <v>0</v>
+      <c r="D7" s="71" t="n">
+        <v>144000</v>
       </c>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="n"/>
+      <c r="E7" s="71" t="n">
+        <v>144000</v>
+      </c>
+      <c r="F7" s="71" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G7" s="71" t="n">
+        <v>360000</v>
+      </c>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
       <c r="J7" s="1" t="n"/>
@@ -29319,7 +29342,7 @@
     </row>
     <row r="8" ht="22" customHeight="1" s="43">
       <c r="A8" s="1" t="n"/>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="72" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="59" t="inlineStr">
@@ -29327,12 +29350,18 @@
           <t>Travel</t>
         </is>
       </c>
-      <c r="D8" s="74" t="n">
-        <v>0</v>
+      <c r="D8" s="73" t="n">
+        <v>50000</v>
       </c>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
+      <c r="E8" s="73" t="n">
+        <v>90000</v>
+      </c>
+      <c r="F8" s="73" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G8" s="73" t="n">
+        <v>200000</v>
+      </c>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
       <c r="J8" s="1" t="n"/>
@@ -29355,7 +29384,7 @@
     </row>
     <row r="9" ht="22" customHeight="1" s="43">
       <c r="A9" s="1" t="n"/>
-      <c r="B9" s="71" t="n">
+      <c r="B9" s="70" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="61" t="inlineStr">
@@ -29363,12 +29392,18 @@
           <t>Miscellaneous expenses</t>
         </is>
       </c>
-      <c r="D9" s="72" t="n">
-        <v>0</v>
+      <c r="D9" s="71" t="n">
+        <v>100000</v>
       </c>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
+      <c r="E9" s="71" t="n">
+        <v>160000</v>
+      </c>
+      <c r="F9" s="71" t="n">
+        <v>180000</v>
+      </c>
+      <c r="G9" s="71" t="n">
+        <v>440000</v>
+      </c>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
       <c r="J9" s="1" t="n"/>
@@ -29391,7 +29426,7 @@
     </row>
     <row r="10" ht="22" customHeight="1" s="43">
       <c r="A10" s="1" t="n"/>
-      <c r="B10" s="73" t="n">
+      <c r="B10" s="72" t="n">
         <v>6</v>
       </c>
       <c r="C10" s="59" t="inlineStr">
@@ -29399,12 +29434,18 @@
           <t>Contingency (max 5%)</t>
         </is>
       </c>
-      <c r="D10" s="74" t="n">
-        <v>780</v>
+      <c r="D10" s="73" t="n">
+        <v>50700</v>
       </c>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="n"/>
-      <c r="G10" s="1" t="n"/>
+      <c r="E10" s="73" t="n">
+        <v>55700</v>
+      </c>
+      <c r="F10" s="73" t="n">
+        <v>33600</v>
+      </c>
+      <c r="G10" s="73" t="n">
+        <v>140000</v>
+      </c>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
       <c r="J10" s="1" t="n"/>
@@ -29427,7 +29468,7 @@
     </row>
     <row r="11" ht="22" customHeight="1" s="43">
       <c r="A11" s="1" t="n"/>
-      <c r="B11" s="75" t="n">
+      <c r="B11" s="74" t="n">
         <v>7</v>
       </c>
       <c r="C11" s="63" t="inlineStr">
@@ -29435,12 +29476,18 @@
           <t>Sub total</t>
         </is>
       </c>
-      <c r="D11" s="76" t="n">
-        <v>16380</v>
+      <c r="D11" s="75" t="n">
+        <v>1064700</v>
       </c>
-      <c r="E11" s="1" t="n"/>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
+      <c r="E11" s="75" t="n">
+        <v>1169700</v>
+      </c>
+      <c r="F11" s="75" t="n">
+        <v>705600</v>
+      </c>
+      <c r="G11" s="75" t="n">
+        <v>2940000</v>
+      </c>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
       <c r="J11" s="1" t="n"/>
@@ -29463,7 +29510,7 @@
     </row>
     <row r="12" ht="22" customHeight="1" s="43">
       <c r="A12" s="1" t="n"/>
-      <c r="B12" s="73" t="n">
+      <c r="B12" s="72" t="n">
         <v>8</v>
       </c>
       <c r="C12" s="59" t="inlineStr">
@@ -29471,12 +29518,18 @@
           <t>Overhead (max 20%)</t>
         </is>
       </c>
-      <c r="D12" s="74" t="n">
-        <v>3276</v>
+      <c r="D12" s="73" t="n">
+        <v>212940</v>
       </c>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
+      <c r="E12" s="73" t="n">
+        <v>233940</v>
+      </c>
+      <c r="F12" s="73" t="n">
+        <v>141120</v>
+      </c>
+      <c r="G12" s="73" t="n">
+        <v>588000</v>
+      </c>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
       <c r="J12" s="1" t="n"/>
@@ -29499,7 +29552,7 @@
     </row>
     <row r="13" ht="22" customHeight="1" s="43">
       <c r="A13" s="1" t="n"/>
-      <c r="B13" s="71" t="n">
+      <c r="B13" s="70" t="n">
         <v>9</v>
       </c>
       <c r="C13" s="61" t="inlineStr">
@@ -29507,12 +29560,18 @@
           <t>Faculty fee (max 20%)</t>
         </is>
       </c>
-      <c r="D13" s="72" t="n">
-        <v>3931</v>
+      <c r="D13" s="71" t="n">
+        <v>255528</v>
       </c>
-      <c r="E13" s="1" t="n"/>
-      <c r="F13" s="1" t="n"/>
-      <c r="G13" s="1" t="n"/>
+      <c r="E13" s="71" t="n">
+        <v>280728</v>
+      </c>
+      <c r="F13" s="71" t="n">
+        <v>169344</v>
+      </c>
+      <c r="G13" s="71" t="n">
+        <v>705600</v>
+      </c>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
       <c r="J13" s="1" t="n"/>
@@ -29535,7 +29594,7 @@
     </row>
     <row r="14" ht="22" customHeight="1" s="43">
       <c r="A14" s="1" t="n"/>
-      <c r="B14" s="77" t="n">
+      <c r="B14" s="76" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="65" t="inlineStr">
@@ -29543,12 +29602,18 @@
           <t>Total (7+8+9)</t>
         </is>
       </c>
-      <c r="D14" s="78" t="n">
-        <v>23587</v>
+      <c r="D14" s="77" t="n">
+        <v>1533168</v>
       </c>
-      <c r="E14" s="1" t="n"/>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
+      <c r="E14" s="77" t="n">
+        <v>1684368</v>
+      </c>
+      <c r="F14" s="77" t="n">
+        <v>1016064</v>
+      </c>
+      <c r="G14" s="77" t="n">
+        <v>4233600</v>
+      </c>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
       <c r="J14" s="1" t="n"/>
@@ -29571,7 +29636,7 @@
     </row>
     <row r="15" ht="22" customHeight="1" s="43">
       <c r="A15" s="1" t="n"/>
-      <c r="B15" s="71" t="n">
+      <c r="B15" s="70" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="61" t="inlineStr">
@@ -29579,12 +29644,18 @@
           <t>GST (18% of 10)</t>
         </is>
       </c>
-      <c r="D15" s="72" t="n">
+      <c r="D15" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="1" t="n"/>
-      <c r="F15" s="1" t="n"/>
-      <c r="G15" s="1" t="n"/>
+      <c r="E15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="71" t="n">
+        <v>0</v>
+      </c>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
       <c r="J15" s="1" t="n"/>
@@ -29607,7 +29678,7 @@
     </row>
     <row r="16" ht="22" customHeight="1" s="43">
       <c r="A16" s="1" t="n"/>
-      <c r="B16" s="77" t="n">
+      <c r="B16" s="76" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="65" t="inlineStr">
@@ -29615,12 +29686,18 @@
           <t>Grand total (10+11)</t>
         </is>
       </c>
-      <c r="D16" s="78" t="n">
-        <v>23587</v>
+      <c r="D16" s="77" t="n">
+        <v>1533168</v>
       </c>
-      <c r="E16" s="79" t="n"/>
-      <c r="F16" s="79" t="n"/>
-      <c r="G16" s="1" t="n"/>
+      <c r="E16" s="77" t="n">
+        <v>1684368</v>
+      </c>
+      <c r="F16" s="77" t="n">
+        <v>1016064</v>
+      </c>
+      <c r="G16" s="77" t="n">
+        <v>4233600</v>
+      </c>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
@@ -29643,11 +29720,11 @@
     </row>
     <row r="17" ht="14.25" customHeight="1" s="43">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="79" t="n"/>
-      <c r="C17" s="79" t="n"/>
-      <c r="D17" s="79" t="n"/>
-      <c r="E17" s="79" t="n"/>
-      <c r="F17" s="79" t="n"/>
+      <c r="B17" s="78" t="n"/>
+      <c r="C17" s="78" t="n"/>
+      <c r="D17" s="78" t="n"/>
+      <c r="E17" s="78" t="n"/>
+      <c r="F17" s="78" t="n"/>
       <c r="G17" s="1" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
@@ -29671,12 +29748,11 @@
     </row>
     <row r="18" ht="30" customHeight="1" s="43">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="80" t="inlineStr">
+      <c r="B18" s="79" t="inlineStr">
         <is>
-          <t>80 percent of each tranche is spent before the next is claimed. Tranche amounts are set out on the Milestones sheet.</t>
+          <t>80 percent of each tranche is spent before the next is claimed. Prototype parts to date (INR 23,587) were invested before T0 and are not part of this request.</t>
         </is>
       </c>
-      <c r="G18" s="1" t="n"/>
       <c r="H18" s="1" t="n"/>
       <c r="I18" s="1" t="n"/>
       <c r="J18" s="1" t="n"/>
@@ -57251,12 +57327,12 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(office): cap the faculty fee at 3 lakh and move the balance into R&D
The faculty fee was 7.06 lakh at the 20 percent cap. It is now 3.00 lakh, and the released amount buys equipment and consumables: reference instruments for the R&D bench (2.4 lakh) and five more pilot sets (0.8 lakh).

Because contingency and overhead are percentages, redirecting the fee also moves those two heads. The grand total falls by 2,400 to 42,31,200, and the tranches are recomputed so every head still sums across the three phases.
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="K4" s="60" t="n">
-        <v>1533168</v>
+        <v>1569160</v>
       </c>
       <c r="L4" s="59" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="C5" s="62" t="n">
-        <v>600000</v>
+        <v>840000</v>
       </c>
       <c r="E5" s="61" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="H5" s="61" t="inlineStr">
         <is>
-          <t>20 sets, IP68 and EMC passed</t>
+          <t>25 sets, IP68 and EMC passed</t>
         </is>
       </c>
       <c r="J5" s="61" t="inlineStr">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="K5" s="62" t="n">
-        <v>1684368</v>
+        <v>1639560</v>
       </c>
       <c r="L5" s="61" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="C6" s="60" t="n">
-        <v>360000</v>
+        <v>440000</v>
       </c>
       <c r="E6" s="59" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="K6" s="60" t="n">
-        <v>1016064</v>
+        <v>1022480</v>
       </c>
       <c r="L6" s="59" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="K7" s="64" t="n">
-        <v>4233600</v>
+        <v>4231200</v>
       </c>
       <c r="L7" s="63" t="inlineStr"/>
       <c r="M7" s="12" t="n"/>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="C9" s="62" t="n">
-        <v>140000</v>
+        <v>156000</v>
       </c>
       <c r="E9" s="36" t="n"/>
       <c r="F9" s="36" t="n"/>
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="C10" s="67" t="n">
-        <v>2940000</v>
+        <v>3276000</v>
       </c>
       <c r="E10" s="36" t="n"/>
       <c r="F10" s="37" t="n"/>
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C11" s="62" t="n">
-        <v>588000</v>
+        <v>655200</v>
       </c>
       <c r="E11" s="40" t="n"/>
       <c r="F11" s="12" t="n"/>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="C12" s="60" t="n">
-        <v>705600</v>
+        <v>300000</v>
       </c>
       <c r="E12" s="40" t="n"/>
       <c r="F12" s="12" t="n"/>
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="C13" s="64" t="n">
-        <v>4233600</v>
+        <v>4231200</v>
       </c>
       <c r="E13" s="40" t="n"/>
       <c r="F13" s="12" t="n"/>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="C15" s="64" t="n">
-        <v>4233600</v>
+        <v>4231200</v>
       </c>
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="12" t="n"/>
@@ -29139,7 +29139,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="69" t="inlineStr">
         <is>
-          <t>Grant total: INR 42,33,600</t>
+          <t>Grant total: INR 42,31,200</t>
         </is>
       </c>
       <c r="H3" s="1" t="n"/>
@@ -29267,16 +29267,16 @@
         </is>
       </c>
       <c r="D6" s="73" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="E6" s="73" t="n">
-        <v>240000</v>
+        <v>300000</v>
       </c>
       <c r="F6" s="73" t="n">
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="G6" s="73" t="n">
-        <v>600000</v>
+        <v>840000</v>
       </c>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
@@ -29309,16 +29309,16 @@
         </is>
       </c>
       <c r="D7" s="71" t="n">
-        <v>144000</v>
+        <v>176000</v>
       </c>
       <c r="E7" s="71" t="n">
-        <v>144000</v>
+        <v>176000</v>
       </c>
       <c r="F7" s="71" t="n">
-        <v>72000</v>
+        <v>88000</v>
       </c>
       <c r="G7" s="71" t="n">
-        <v>360000</v>
+        <v>440000</v>
       </c>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
@@ -29435,16 +29435,16 @@
         </is>
       </c>
       <c r="D10" s="73" t="n">
-        <v>50700</v>
+        <v>58300</v>
       </c>
       <c r="E10" s="73" t="n">
-        <v>55700</v>
+        <v>60300</v>
       </c>
       <c r="F10" s="73" t="n">
-        <v>33600</v>
+        <v>37400</v>
       </c>
       <c r="G10" s="73" t="n">
-        <v>140000</v>
+        <v>156000</v>
       </c>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
@@ -29477,16 +29477,16 @@
         </is>
       </c>
       <c r="D11" s="75" t="n">
-        <v>1064700</v>
+        <v>1224300</v>
       </c>
       <c r="E11" s="75" t="n">
-        <v>1169700</v>
+        <v>1266300</v>
       </c>
       <c r="F11" s="75" t="n">
-        <v>705600</v>
+        <v>785400</v>
       </c>
       <c r="G11" s="75" t="n">
-        <v>2940000</v>
+        <v>3276000</v>
       </c>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
@@ -29519,16 +29519,16 @@
         </is>
       </c>
       <c r="D12" s="73" t="n">
-        <v>212940</v>
+        <v>244860</v>
       </c>
       <c r="E12" s="73" t="n">
-        <v>233940</v>
+        <v>253260</v>
       </c>
       <c r="F12" s="73" t="n">
-        <v>141120</v>
+        <v>157080</v>
       </c>
       <c r="G12" s="73" t="n">
-        <v>588000</v>
+        <v>655200</v>
       </c>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
@@ -29561,16 +29561,16 @@
         </is>
       </c>
       <c r="D13" s="71" t="n">
-        <v>255528</v>
+        <v>100000</v>
       </c>
       <c r="E13" s="71" t="n">
-        <v>280728</v>
+        <v>120000</v>
       </c>
       <c r="F13" s="71" t="n">
-        <v>169344</v>
+        <v>80000</v>
       </c>
       <c r="G13" s="71" t="n">
-        <v>705600</v>
+        <v>300000</v>
       </c>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
@@ -29603,16 +29603,16 @@
         </is>
       </c>
       <c r="D14" s="77" t="n">
-        <v>1533168</v>
+        <v>1569160</v>
       </c>
       <c r="E14" s="77" t="n">
-        <v>1684368</v>
+        <v>1639560</v>
       </c>
       <c r="F14" s="77" t="n">
-        <v>1016064</v>
+        <v>1022480</v>
       </c>
       <c r="G14" s="77" t="n">
-        <v>4233600</v>
+        <v>4231200</v>
       </c>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
@@ -29687,16 +29687,16 @@
         </is>
       </c>
       <c r="D16" s="77" t="n">
-        <v>1533168</v>
+        <v>1569160</v>
       </c>
       <c r="E16" s="77" t="n">
-        <v>1684368</v>
+        <v>1639560</v>
       </c>
       <c r="F16" s="77" t="n">
-        <v>1016064</v>
+        <v>1022480</v>
       </c>
       <c r="G16" s="77" t="n">
-        <v>4233600</v>
+        <v>4231200</v>
       </c>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>

</xml_diff>

<commit_message>
docs(office): add the institute logos, set the Water Management theme, and make costs GST-inclusive
The cover now carries the TIH and IIT Bombay marks with the foundation's contact strip, composed into one band and placed in the first-page footer so Word renders it reliably.

The theme field reads Water Management. The history section is now a 185-word review of five prior studies: tank monitoring on ESP32 and ESP8266, and the Gazebo-only cleaning robot. The objectives open with an 81-word statement of the gap against that work.

Every cost line is now labelled inclusive of GST, in the proposal, the deck and the workbook.
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -821,7 +821,7 @@
   <cols>
     <col width="7" customWidth="1" style="43" min="1" max="1"/>
     <col width="29" customWidth="1" style="43" min="2" max="2"/>
-    <col width="13" customWidth="1" style="43" min="3" max="3"/>
+    <col width="16" customWidth="1" style="43" min="3" max="3"/>
     <col width="2.5" customWidth="1" style="43" min="4" max="4"/>
     <col width="5.5" customWidth="1" style="43" min="5" max="5"/>
     <col width="31" customWidth="1" style="43" min="6" max="6"/>
@@ -886,7 +886,7 @@
       <c r="Y2" s="12" t="n"/>
       <c r="Z2" s="12" t="n"/>
     </row>
-    <row r="3" ht="34" customHeight="1" s="43">
+    <row r="3" ht="40" customHeight="1" s="43">
       <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Sr. No.</t>
@@ -899,7 +899,7 @@
       </c>
       <c r="C3" s="58" t="inlineStr">
         <is>
-          <t>Total (Rs.)</t>
+          <t>Total (Rs., incl. GST)</t>
         </is>
       </c>
       <c r="E3" s="58" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B5" s="61" t="inlineStr">
         <is>
-          <t>Equipment (exclusive of GST)</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="C5" s="62" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>GST (18% of 10)</t>
+          <t>GST (18%, included)</t>
         </is>
       </c>
       <c r="C14" s="60" t="n">
@@ -29191,7 +29191,7 @@
       </c>
       <c r="G4" s="58" t="inlineStr">
         <is>
-          <t>Total (INR)</t>
+          <t>Total (INR, incl. GST)</t>
         </is>
       </c>
       <c r="H4" s="1" t="n"/>
@@ -29263,7 +29263,7 @@
       </c>
       <c r="C6" s="59" t="inlineStr">
         <is>
-          <t>Equipment (exclusive of GST)</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="D6" s="73" t="n">
@@ -29641,7 +29641,7 @@
       </c>
       <c r="C15" s="61" t="inlineStr">
         <is>
-          <t>GST (18% of 10)</t>
+          <t>GST (18%, included)</t>
         </is>
       </c>
       <c r="D15" s="71" t="n">
@@ -29750,7 +29750,7 @@
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="79" t="inlineStr">
         <is>
-          <t>80 percent of each tranche is spent before the next is claimed. Prototype parts to date (INR 23,587) were invested before T0 and are not part of this request.</t>
+          <t>80 percent of each tranche is spent before the next is claimed. All figures include GST at 18 percent. Prototype parts to date (INR 23,587) were invested before T0 and are not part of this request.</t>
         </is>
       </c>
       <c r="H18" s="1" t="n"/>

</xml_diff>

<commit_message>
docs: rebuild the grant around the 47 lakh pilot-line budget
The equipment head is now the pilot line itself: a used 100 T moulder, three moulds, a stencil printer, a two-head PnP, a six-zone reflow and the test bench, itemised across 17 lines.

Heads: equipment 24,27,288, manpower 7,20,000, consumables 3,40,000, travel 1,00,000, misc 17,966, contingency 1,80,263, faculty 2,00,000, GST 7,17,393. Total 47,02,910, 94 percent of the ceiling.

Tranches follow the spend: 25,66,222 at T0, 16,23,623 at month 6, 5,13,065 at month 12. Milestone 1 becomes line procurement, and the proposal gains a 4.2 equipment breakdown; the workbook gains an Equipment sheet.

The C1 controller is an ESP8266, so the appendix and the specification no longer call it an ESP32.
</commit_message>
<xml_diff>
--- a/docs/office/TankGuard_Budget_Milestone.xlsx
+++ b/docs/office/TankGuard_Budget_Milestone.xlsx
@@ -5,10 +5,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Milestones'!$A$1:$L$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Budget'!$B$2:$G$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Equipment'!$B$2:$D$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -108,6 +110,12 @@
       <i val="1"/>
       <color rgb="00404040"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -346,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -540,6 +548,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -899,7 +910,7 @@
       </c>
       <c r="C3" s="58" t="inlineStr">
         <is>
-          <t>Total (Rs., incl. GST)</t>
+          <t>Total (Rs.)</t>
         </is>
       </c>
       <c r="E3" s="58" t="inlineStr">
@@ -962,7 +973,7 @@
         </is>
       </c>
       <c r="C4" s="60" t="n">
-        <v>1200000</v>
+        <v>720000</v>
       </c>
       <c r="E4" s="59" t="inlineStr">
         <is>
@@ -971,7 +982,7 @@
       </c>
       <c r="F4" s="59" t="inlineStr">
         <is>
-          <t>Milestone 1: Design freeze and tooling</t>
+          <t>Milestone 1: Design freeze and line procurement</t>
         </is>
       </c>
       <c r="G4" s="59" t="inlineStr">
@@ -981,7 +992,7 @@
       </c>
       <c r="H4" s="59" t="inlineStr">
         <is>
-          <t>Moulds ordered, 5 pilot sets built</t>
+          <t>Line installed, design frozen</t>
         </is>
       </c>
       <c r="J4" s="59" t="inlineStr">
@@ -990,11 +1001,11 @@
         </is>
       </c>
       <c r="K4" s="60" t="n">
-        <v>1569160</v>
+        <v>2566222</v>
       </c>
       <c r="L4" s="59" t="inlineStr">
         <is>
-          <t>Design freeze, tooling, first pilot sets</t>
+          <t>Line procurement, tooling, design freeze</t>
         </is>
       </c>
       <c r="M4" s="12" t="n"/>
@@ -1022,7 +1033,7 @@
         </is>
       </c>
       <c r="C5" s="62" t="n">
-        <v>840000</v>
+        <v>2427288</v>
       </c>
       <c r="E5" s="61" t="inlineStr">
         <is>
@@ -1050,7 +1061,7 @@
         </is>
       </c>
       <c r="K5" s="62" t="n">
-        <v>1639560</v>
+        <v>1623623</v>
       </c>
       <c r="L5" s="61" t="inlineStr">
         <is>
@@ -1082,7 +1093,7 @@
         </is>
       </c>
       <c r="C6" s="60" t="n">
-        <v>440000</v>
+        <v>340000</v>
       </c>
       <c r="E6" s="59" t="inlineStr">
         <is>
@@ -1110,7 +1121,7 @@
         </is>
       </c>
       <c r="K6" s="60" t="n">
-        <v>1022480</v>
+        <v>513065</v>
       </c>
       <c r="L6" s="59" t="inlineStr">
         <is>
@@ -1142,7 +1153,7 @@
         </is>
       </c>
       <c r="C7" s="62" t="n">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="E7" s="61" t="inlineStr">
         <is>
@@ -1170,7 +1181,7 @@
         </is>
       </c>
       <c r="K7" s="64" t="n">
-        <v>4231200</v>
+        <v>4702910</v>
       </c>
       <c r="L7" s="63" t="inlineStr"/>
       <c r="M7" s="12" t="n"/>
@@ -1198,7 +1209,7 @@
         </is>
       </c>
       <c r="C8" s="60" t="n">
-        <v>440000</v>
+        <v>17966</v>
       </c>
       <c r="E8" s="65" t="n"/>
       <c r="F8" s="65" t="inlineStr">
@@ -1236,7 +1247,7 @@
         </is>
       </c>
       <c r="C9" s="62" t="n">
-        <v>156000</v>
+        <v>180263</v>
       </c>
       <c r="E9" s="36" t="n"/>
       <c r="F9" s="36" t="n"/>
@@ -1269,7 +1280,7 @@
         </is>
       </c>
       <c r="C10" s="67" t="n">
-        <v>3276000</v>
+        <v>3785517</v>
       </c>
       <c r="E10" s="36" t="n"/>
       <c r="F10" s="37" t="n"/>
@@ -1304,7 +1315,7 @@
         </is>
       </c>
       <c r="C11" s="62" t="n">
-        <v>655200</v>
+        <v>0</v>
       </c>
       <c r="E11" s="40" t="n"/>
       <c r="F11" s="12" t="n"/>
@@ -1335,11 +1346,11 @@
       </c>
       <c r="B12" s="59" t="inlineStr">
         <is>
-          <t>Faculty fee (max 20%)</t>
+          <t>Faculty fee</t>
         </is>
       </c>
       <c r="C12" s="60" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="E12" s="40" t="n"/>
       <c r="F12" s="12" t="n"/>
@@ -1374,7 +1385,7 @@
         </is>
       </c>
       <c r="C13" s="64" t="n">
-        <v>4231200</v>
+        <v>3985517</v>
       </c>
       <c r="E13" s="40" t="n"/>
       <c r="F13" s="12" t="n"/>
@@ -1405,11 +1416,11 @@
       </c>
       <c r="B14" s="59" t="inlineStr">
         <is>
-          <t>GST (18%, included)</t>
+          <t>GST (18%)</t>
         </is>
       </c>
       <c r="C14" s="60" t="n">
-        <v>0</v>
+        <v>717393</v>
       </c>
       <c r="E14" s="12" t="n"/>
       <c r="F14" s="12" t="n"/>
@@ -1444,7 +1455,7 @@
         </is>
       </c>
       <c r="C15" s="64" t="n">
-        <v>4231200</v>
+        <v>4702910</v>
       </c>
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="12" t="n"/>
@@ -29191,7 +29202,7 @@
       </c>
       <c r="G4" s="58" t="inlineStr">
         <is>
-          <t>Total (INR, incl. GST)</t>
+          <t>Total (INR)</t>
         </is>
       </c>
       <c r="H4" s="1" t="n"/>
@@ -29225,16 +29236,16 @@
         </is>
       </c>
       <c r="D5" s="71" t="n">
-        <v>360000</v>
+        <v>240000</v>
       </c>
       <c r="E5" s="71" t="n">
-        <v>480000</v>
+        <v>240000</v>
       </c>
       <c r="F5" s="71" t="n">
-        <v>360000</v>
+        <v>240000</v>
       </c>
       <c r="G5" s="71" t="n">
-        <v>1200000</v>
+        <v>720000</v>
       </c>
       <c r="H5" s="1" t="n"/>
       <c r="I5" s="1" t="n"/>
@@ -29267,16 +29278,16 @@
         </is>
       </c>
       <c r="D6" s="73" t="n">
-        <v>480000</v>
+        <v>1600000</v>
       </c>
       <c r="E6" s="73" t="n">
-        <v>300000</v>
+        <v>827288</v>
       </c>
       <c r="F6" s="73" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="73" t="n">
-        <v>840000</v>
+        <v>2427288</v>
       </c>
       <c r="H6" s="1" t="n"/>
       <c r="I6" s="1" t="n"/>
@@ -29309,16 +29320,16 @@
         </is>
       </c>
       <c r="D7" s="71" t="n">
-        <v>176000</v>
+        <v>100000</v>
       </c>
       <c r="E7" s="71" t="n">
-        <v>176000</v>
+        <v>140000</v>
       </c>
       <c r="F7" s="71" t="n">
-        <v>88000</v>
+        <v>100000</v>
       </c>
       <c r="G7" s="71" t="n">
-        <v>440000</v>
+        <v>340000</v>
       </c>
       <c r="H7" s="1" t="n"/>
       <c r="I7" s="1" t="n"/>
@@ -29351,16 +29362,16 @@
         </is>
       </c>
       <c r="D8" s="73" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="E8" s="73" t="n">
-        <v>90000</v>
+        <v>40000</v>
       </c>
       <c r="F8" s="73" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="G8" s="73" t="n">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="H8" s="1" t="n"/>
       <c r="I8" s="1" t="n"/>
@@ -29393,16 +29404,16 @@
         </is>
       </c>
       <c r="D9" s="71" t="n">
-        <v>100000</v>
+        <v>5966</v>
       </c>
       <c r="E9" s="71" t="n">
-        <v>160000</v>
+        <v>6000</v>
       </c>
       <c r="F9" s="71" t="n">
-        <v>180000</v>
+        <v>6000</v>
       </c>
       <c r="G9" s="71" t="n">
-        <v>440000</v>
+        <v>17966</v>
       </c>
       <c r="H9" s="1" t="n"/>
       <c r="I9" s="1" t="n"/>
@@ -29435,16 +29446,16 @@
         </is>
       </c>
       <c r="D10" s="73" t="n">
-        <v>58300</v>
+        <v>98798</v>
       </c>
       <c r="E10" s="73" t="n">
-        <v>60300</v>
+        <v>62664</v>
       </c>
       <c r="F10" s="73" t="n">
-        <v>37400</v>
+        <v>18801</v>
       </c>
       <c r="G10" s="73" t="n">
-        <v>156000</v>
+        <v>180263</v>
       </c>
       <c r="H10" s="1" t="n"/>
       <c r="I10" s="1" t="n"/>
@@ -29477,16 +29488,16 @@
         </is>
       </c>
       <c r="D11" s="75" t="n">
-        <v>1224300</v>
+        <v>2074764</v>
       </c>
       <c r="E11" s="75" t="n">
-        <v>1266300</v>
+        <v>1315952</v>
       </c>
       <c r="F11" s="75" t="n">
-        <v>785400</v>
+        <v>394801</v>
       </c>
       <c r="G11" s="75" t="n">
-        <v>3276000</v>
+        <v>3785517</v>
       </c>
       <c r="H11" s="1" t="n"/>
       <c r="I11" s="1" t="n"/>
@@ -29519,16 +29530,16 @@
         </is>
       </c>
       <c r="D12" s="73" t="n">
-        <v>244860</v>
+        <v>0</v>
       </c>
       <c r="E12" s="73" t="n">
-        <v>253260</v>
+        <v>0</v>
       </c>
       <c r="F12" s="73" t="n">
-        <v>157080</v>
+        <v>0</v>
       </c>
       <c r="G12" s="73" t="n">
-        <v>655200</v>
+        <v>0</v>
       </c>
       <c r="H12" s="1" t="n"/>
       <c r="I12" s="1" t="n"/>
@@ -29557,20 +29568,20 @@
       </c>
       <c r="C13" s="61" t="inlineStr">
         <is>
-          <t>Faculty fee (max 20%)</t>
+          <t>Faculty fee</t>
         </is>
       </c>
       <c r="D13" s="71" t="n">
         <v>100000</v>
       </c>
       <c r="E13" s="71" t="n">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="F13" s="71" t="n">
-        <v>80000</v>
+        <v>40000</v>
       </c>
       <c r="G13" s="71" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="H13" s="1" t="n"/>
       <c r="I13" s="1" t="n"/>
@@ -29603,16 +29614,16 @@
         </is>
       </c>
       <c r="D14" s="77" t="n">
-        <v>1569160</v>
+        <v>2174764</v>
       </c>
       <c r="E14" s="77" t="n">
-        <v>1639560</v>
+        <v>1375952</v>
       </c>
       <c r="F14" s="77" t="n">
-        <v>1022480</v>
+        <v>434801</v>
       </c>
       <c r="G14" s="77" t="n">
-        <v>4231200</v>
+        <v>3985517</v>
       </c>
       <c r="H14" s="1" t="n"/>
       <c r="I14" s="1" t="n"/>
@@ -29641,20 +29652,20 @@
       </c>
       <c r="C15" s="61" t="inlineStr">
         <is>
-          <t>GST (18%, included)</t>
+          <t>GST (18%)</t>
         </is>
       </c>
       <c r="D15" s="71" t="n">
-        <v>0</v>
+        <v>391458</v>
       </c>
       <c r="E15" s="71" t="n">
-        <v>0</v>
+        <v>247671</v>
       </c>
       <c r="F15" s="71" t="n">
-        <v>0</v>
+        <v>78264</v>
       </c>
       <c r="G15" s="71" t="n">
-        <v>0</v>
+        <v>717393</v>
       </c>
       <c r="H15" s="1" t="n"/>
       <c r="I15" s="1" t="n"/>
@@ -29687,16 +29698,16 @@
         </is>
       </c>
       <c r="D16" s="77" t="n">
-        <v>1569160</v>
+        <v>2566222</v>
       </c>
       <c r="E16" s="77" t="n">
-        <v>1639560</v>
+        <v>1623623</v>
       </c>
       <c r="F16" s="77" t="n">
-        <v>1022480</v>
+        <v>513065</v>
       </c>
       <c r="G16" s="77" t="n">
-        <v>4231200</v>
+        <v>4702910</v>
       </c>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
@@ -29750,7 +29761,7 @@
       <c r="A18" s="1" t="n"/>
       <c r="B18" s="79" t="inlineStr">
         <is>
-          <t>80 percent of each tranche is spent before the next is claimed. All figures include GST at 18 percent. Prototype parts to date (INR 23,587) were invested before T0 and are not part of this request.</t>
+          <t>80 percent of each tranche is spent before the next is claimed. GST at 18 percent is shown on the total. Prototype parts to date (INR 23,587) were invested before T0 and are not part of this request.</t>
         </is>
       </c>
       <c r="H18" s="1" t="n"/>
@@ -57335,4 +57346,281 @@
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0" footer="0"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="43" min="2" max="2"/>
+    <col width="46" customWidth="1" style="43" min="3" max="3"/>
+    <col width="18" customWidth="1" style="43" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="24" customHeight="1" s="43">
+      <c r="B2" s="68" t="inlineStr">
+        <is>
+          <t>Equipment breakdown - pilot line</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="80" t="inlineStr">
+        <is>
+          <t>Exclusive of GST. Vendor quotes and negotiated targets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Sr. No.</t>
+        </is>
+      </c>
+      <c r="C4" s="58" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t>Amount (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" s="43">
+      <c r="B5" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>Used 100 T injection moulder</t>
+        </is>
+      </c>
+      <c r="D5" s="71" t="n">
+        <v>450000</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" s="43">
+      <c r="B6" s="72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="59" t="inlineStr">
+        <is>
+          <t>Three moulds (toolroom)</t>
+        </is>
+      </c>
+      <c r="D6" s="73" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" s="43">
+      <c r="B7" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>Chiller, dryer, granulator</t>
+        </is>
+      </c>
+      <c r="D7" s="71" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" s="43">
+      <c r="B8" s="72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="59" t="inlineStr">
+        <is>
+          <t>Semi-auto stencil printer</t>
+        </is>
+      </c>
+      <c r="D8" s="73" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="43">
+      <c r="B9" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>Two-head vision pick-and-place</t>
+        </is>
+      </c>
+      <c r="D9" s="71" t="n">
+        <v>310000</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" s="43">
+      <c r="B10" s="72" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>Six-zone reflow oven</t>
+        </is>
+      </c>
+      <c r="D10" s="73" t="n">
+        <v>216500</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" s="43">
+      <c r="B11" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>Rework station</t>
+        </is>
+      </c>
+      <c r="D11" s="71" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" s="43">
+      <c r="B12" s="72" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>Stencils</t>
+        </is>
+      </c>
+      <c r="D12" s="73" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" s="43">
+      <c r="B13" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>Four ESD benches</t>
+        </is>
+      </c>
+      <c r="D13" s="71" t="n">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" s="43">
+      <c r="B14" s="72" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="59" t="inlineStr">
+        <is>
+          <t>Soldering stations and microscope</t>
+        </is>
+      </c>
+      <c r="D14" s="73" t="n">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" s="43">
+      <c r="B15" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>Oscilloscope, PSU, DMM</t>
+        </is>
+      </c>
+      <c r="D15" s="71" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" s="43">
+      <c r="B16" s="72" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>Functional-test fixtures</t>
+        </is>
+      </c>
+      <c r="D16" s="73" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" s="43">
+      <c r="B17" s="70" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="D17" s="71" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" s="43">
+      <c r="B18" s="72" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" s="59" t="inlineStr">
+        <is>
+          <t>Hand tools, crimpers, bench consumables</t>
+        </is>
+      </c>
+      <c r="D18" s="73" t="n">
+        <v>39788</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" s="43">
+      <c r="B19" s="70" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>Electrical, air, fume, fire</t>
+        </is>
+      </c>
+      <c r="D19" s="71" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="43">
+      <c r="B20" s="72" t="n">
+        <v>16</v>
+      </c>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>Freight and installation</t>
+        </is>
+      </c>
+      <c r="D20" s="73" t="n">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="43">
+      <c r="B21" s="74" t="n">
+        <v>17</v>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>Equipment total</t>
+        </is>
+      </c>
+      <c r="D21" s="75" t="n">
+        <v>2427288</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>